<commit_message>
model fix got rid of scenarios
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1374" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2F702C9-63BB-47BC-9507-9427DD99F1FB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="6" activeTab="10" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="10" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -1020,6 +1020,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -2781,6 +2785,26 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -2788,26 +2812,6 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new Scenario Logic
80 Scenarios are created, the instalation of Bess is paused for now, parts that should not be imported are "crossed" out.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1374" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2F702C9-63BB-47BC-9507-9427DD99F1FB}"/>
+  <xr:revisionPtr revIDLastSave="1387" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4F5CACF-96C4-4A92-BECE-A95E104C9789}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="10" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-28920" yWindow="6825" windowWidth="29040" windowHeight="17520" firstSheet="15" activeTab="21" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -2785,26 +2785,6 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -2812,6 +2792,26 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16527,13 +16527,13 @@
         <v>280439.83</v>
       </c>
       <c r="R2">
-        <v>527469.86</v>
+        <v>1</v>
       </c>
       <c r="S2" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T2">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U2">
         <v>1</v>
@@ -16592,13 +16592,13 @@
         <v>274754.90999999997</v>
       </c>
       <c r="R3">
-        <v>516785.56</v>
+        <v>1</v>
       </c>
       <c r="S3" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T3">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U3">
         <v>1</v>
@@ -16657,13 +16657,13 @@
         <v>269179.44</v>
       </c>
       <c r="R4">
-        <v>506302.5</v>
+        <v>1</v>
       </c>
       <c r="S4" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T4">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U4">
         <v>1</v>
@@ -16722,13 +16722,13 @@
         <v>263711.78000000003</v>
       </c>
       <c r="R5">
-        <v>496017.89</v>
+        <v>1</v>
       </c>
       <c r="S5" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T5">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U5">
         <v>1</v>
@@ -16787,13 +16787,13 @@
         <v>258350.32</v>
       </c>
       <c r="R6">
-        <v>485929.01</v>
+        <v>1</v>
       </c>
       <c r="S6" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T6">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U6">
         <v>1</v>
@@ -16852,13 +16852,13 @@
         <v>253093.46</v>
       </c>
       <c r="R7">
-        <v>476033.18</v>
+        <v>1</v>
       </c>
       <c r="S7" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T7">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U7">
         <v>1</v>
@@ -16917,13 +16917,13 @@
         <v>247939.65</v>
       </c>
       <c r="R8">
-        <v>466327.8</v>
+        <v>1</v>
       </c>
       <c r="S8" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T8">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U8">
         <v>1</v>
@@ -16982,13 +16982,13 @@
         <v>242887.37</v>
       </c>
       <c r="R9">
-        <v>456810.3</v>
+        <v>1</v>
       </c>
       <c r="S9" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T9">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U9">
         <v>1</v>
@@ -17047,13 +17047,13 @@
         <v>237935.1</v>
       </c>
       <c r="R10">
-        <v>447478.16</v>
+        <v>1</v>
       </c>
       <c r="S10" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T10">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U10">
         <v>1</v>
@@ -17112,13 +17112,13 @@
         <v>233081.4</v>
       </c>
       <c r="R11">
-        <v>438328.91</v>
+        <v>1</v>
       </c>
       <c r="S11" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T11">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U11">
         <v>1</v>
@@ -17177,13 +17177,13 @@
         <v>228324.82</v>
       </c>
       <c r="R12">
-        <v>429360.14</v>
+        <v>1</v>
       </c>
       <c r="S12" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T12">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U12">
         <v>1</v>
@@ -17242,13 +17242,13 @@
         <v>223663.91</v>
       </c>
       <c r="R13">
-        <v>420569.49</v>
+        <v>1</v>
       </c>
       <c r="S13" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T13">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U13">
         <v>1</v>
@@ -17307,13 +17307,13 @@
         <v>219097.32</v>
       </c>
       <c r="R14">
-        <v>411954.65</v>
+        <v>1</v>
       </c>
       <c r="S14" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T14">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U14">
         <v>1</v>
@@ -17372,13 +17372,13 @@
         <v>214623.65</v>
       </c>
       <c r="R15">
-        <v>403513.36</v>
+        <v>1</v>
       </c>
       <c r="S15" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T15">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U15">
         <v>1</v>
@@ -17437,13 +17437,13 @@
         <v>210241.6</v>
       </c>
       <c r="R16">
-        <v>395243.39</v>
+        <v>1</v>
       </c>
       <c r="S16" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T16">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U16">
         <v>1</v>
@@ -17502,13 +17502,13 @@
         <v>205949.84</v>
       </c>
       <c r="R17">
-        <v>387142.59</v>
+        <v>1</v>
       </c>
       <c r="S17" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T17">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U17">
         <v>1</v>
@@ -17567,13 +17567,13 @@
         <v>201747.12</v>
       </c>
       <c r="R18">
-        <v>379208.83</v>
+        <v>1</v>
       </c>
       <c r="S18" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T18">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U18">
         <v>1</v>
@@ -17632,13 +17632,13 @@
         <v>197632.19</v>
       </c>
       <c r="R19">
-        <v>371440.05</v>
+        <v>1</v>
       </c>
       <c r="S19" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T19">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U19">
         <v>1</v>
@@ -17697,13 +17697,13 @@
         <v>193603.83</v>
       </c>
       <c r="R20">
-        <v>363834.24</v>
+        <v>1</v>
       </c>
       <c r="S20" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T20">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U20">
         <v>1</v>
@@ -17762,13 +17762,13 @@
         <v>189660.87</v>
       </c>
       <c r="R21">
-        <v>356389.41</v>
+        <v>1</v>
       </c>
       <c r="S21" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T21">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U21">
         <v>1</v>
@@ -17827,13 +17827,13 @@
         <v>185802.14</v>
       </c>
       <c r="R22">
-        <v>349103.66</v>
+        <v>1</v>
       </c>
       <c r="S22" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T22">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U22">
         <v>1</v>
@@ -17892,13 +17892,13 @@
         <v>182026.51</v>
       </c>
       <c r="R23">
-        <v>341975.1</v>
+        <v>1</v>
       </c>
       <c r="S23" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T23">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U23">
         <v>1</v>
@@ -17957,13 +17957,13 @@
         <v>178332.87</v>
       </c>
       <c r="R24">
-        <v>334991.90000000002</v>
+        <v>1</v>
       </c>
       <c r="S24" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T24">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U24">
         <v>1</v>
@@ -18022,13 +18022,13 @@
         <v>174720.11</v>
       </c>
       <c r="R25">
-        <v>328152.28999999998</v>
+        <v>1</v>
       </c>
       <c r="S25" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T25">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U25">
         <v>1</v>
@@ -18087,13 +18087,13 @@
         <v>171187.17</v>
       </c>
       <c r="R26">
-        <v>321454.53999999998</v>
+        <v>1</v>
       </c>
       <c r="S26" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T26">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U26">
         <v>1</v>
@@ -18152,13 +18152,13 @@
         <v>167732.98000000001</v>
       </c>
       <c r="R27">
-        <v>314897</v>
+        <v>1</v>
       </c>
       <c r="S27" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T27">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U27">
         <v>1</v>
@@ -18217,13 +18217,13 @@
         <v>164356.51999999999</v>
       </c>
       <c r="R28">
-        <v>308477.99</v>
+        <v>1</v>
       </c>
       <c r="S28" s="8">
-        <v>519061.86</v>
+        <v>1</v>
       </c>
       <c r="T28">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="U28">
         <v>1</v>
@@ -18789,7 +18789,7 @@
         <v>117</v>
       </c>
       <c r="E14">
-        <v>999999</v>
+        <v>1</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -18902,10 +18902,10 @@
         <v>149960</v>
       </c>
       <c r="F2">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H2">
         <v>382762.9</v>
@@ -18914,10 +18914,10 @@
         <v>679793.6</v>
       </c>
       <c r="J2">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L2">
         <v>479917.1</v>
@@ -18926,7 +18926,7 @@
         <v>787018</v>
       </c>
       <c r="N2">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>280439.83</v>
@@ -18949,10 +18949,10 @@
         <v>148580</v>
       </c>
       <c r="F3">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <v>382762.9</v>
@@ -18961,10 +18961,10 @@
         <v>679793.6</v>
       </c>
       <c r="J3">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K3">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L3">
         <v>479917.1</v>
@@ -18973,7 +18973,7 @@
         <v>787018</v>
       </c>
       <c r="N3">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O3">
         <v>274754.90999999997</v>
@@ -18996,10 +18996,10 @@
         <v>147200</v>
       </c>
       <c r="F4">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H4">
         <v>382762.9</v>
@@ -19008,10 +19008,10 @@
         <v>679793.6</v>
       </c>
       <c r="J4">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K4">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L4">
         <v>479917.1</v>
@@ -19020,7 +19020,7 @@
         <v>787018</v>
       </c>
       <c r="N4">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O4">
         <v>269179.44</v>
@@ -19043,10 +19043,10 @@
         <v>145820</v>
       </c>
       <c r="F5">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H5">
         <v>382762.9</v>
@@ -19055,10 +19055,10 @@
         <v>679793.6</v>
       </c>
       <c r="J5">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K5">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L5">
         <v>479917.1</v>
@@ -19067,7 +19067,7 @@
         <v>787018</v>
       </c>
       <c r="N5">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O5">
         <v>263711.78000000003</v>
@@ -19090,10 +19090,10 @@
         <v>144440</v>
       </c>
       <c r="F6">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H6">
         <v>382762.9</v>
@@ -19102,10 +19102,10 @@
         <v>679793.6</v>
       </c>
       <c r="J6">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K6">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L6">
         <v>479917.1</v>
@@ -19114,7 +19114,7 @@
         <v>787018</v>
       </c>
       <c r="N6">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O6">
         <v>258350.32</v>
@@ -19137,10 +19137,10 @@
         <v>143060</v>
       </c>
       <c r="F7">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H7">
         <v>382762.9</v>
@@ -19149,10 +19149,10 @@
         <v>679793.6</v>
       </c>
       <c r="J7">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L7">
         <v>479917.1</v>
@@ -19161,7 +19161,7 @@
         <v>787018</v>
       </c>
       <c r="N7">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O7">
         <v>253093.46</v>
@@ -19184,10 +19184,10 @@
         <v>141680</v>
       </c>
       <c r="F8">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H8">
         <v>382762.9</v>
@@ -19196,10 +19196,10 @@
         <v>679793.6</v>
       </c>
       <c r="J8">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K8">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L8">
         <v>479917.1</v>
@@ -19208,7 +19208,7 @@
         <v>787018</v>
       </c>
       <c r="N8">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O8">
         <v>247939.65</v>
@@ -19231,10 +19231,10 @@
         <v>140300</v>
       </c>
       <c r="F9">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H9">
         <v>382762.9</v>
@@ -19243,10 +19243,10 @@
         <v>679793.6</v>
       </c>
       <c r="J9">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K9">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L9">
         <v>479917.1</v>
@@ -19255,7 +19255,7 @@
         <v>787018</v>
       </c>
       <c r="N9">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O9">
         <v>242887.37</v>
@@ -19278,10 +19278,10 @@
         <v>138920</v>
       </c>
       <c r="F10">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H10">
         <v>382762.9</v>
@@ -19290,10 +19290,10 @@
         <v>679793.6</v>
       </c>
       <c r="J10">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K10">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L10">
         <v>479917.1</v>
@@ -19302,7 +19302,7 @@
         <v>787018</v>
       </c>
       <c r="N10">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O10">
         <v>237935.1</v>
@@ -19325,10 +19325,10 @@
         <v>137540</v>
       </c>
       <c r="F11">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H11">
         <v>382762.9</v>
@@ -19337,10 +19337,10 @@
         <v>679793.6</v>
       </c>
       <c r="J11">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K11">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L11">
         <v>479917.1</v>
@@ -19349,7 +19349,7 @@
         <v>787018</v>
       </c>
       <c r="N11">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O11">
         <v>233081.4</v>
@@ -19372,10 +19372,10 @@
         <v>136160</v>
       </c>
       <c r="F12">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H12">
         <v>382762.9</v>
@@ -19384,10 +19384,10 @@
         <v>679793.6</v>
       </c>
       <c r="J12">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K12">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L12">
         <v>479917.1</v>
@@ -19396,7 +19396,7 @@
         <v>787018</v>
       </c>
       <c r="N12">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O12">
         <v>228324.82</v>
@@ -19419,10 +19419,10 @@
         <v>134780</v>
       </c>
       <c r="F13">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H13">
         <v>382762.9</v>
@@ -19431,10 +19431,10 @@
         <v>679793.6</v>
       </c>
       <c r="J13">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K13">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L13">
         <v>479917.1</v>
@@ -19443,7 +19443,7 @@
         <v>787018</v>
       </c>
       <c r="N13">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O13">
         <v>223663.91</v>
@@ -19466,10 +19466,10 @@
         <v>133400</v>
       </c>
       <c r="F14">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H14">
         <v>382762.9</v>
@@ -19478,10 +19478,10 @@
         <v>679793.6</v>
       </c>
       <c r="J14">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K14">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L14">
         <v>479917.1</v>
@@ -19490,7 +19490,7 @@
         <v>787018</v>
       </c>
       <c r="N14">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O14">
         <v>219097.32</v>
@@ -19513,10 +19513,10 @@
         <v>132020</v>
       </c>
       <c r="F15">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H15">
         <v>382762.9</v>
@@ -19525,10 +19525,10 @@
         <v>679793.6</v>
       </c>
       <c r="J15">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K15">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L15">
         <v>479917.1</v>
@@ -19537,7 +19537,7 @@
         <v>787018</v>
       </c>
       <c r="N15">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O15">
         <v>214623.65</v>
@@ -19560,10 +19560,10 @@
         <v>130640</v>
       </c>
       <c r="F16">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H16">
         <v>382762.9</v>
@@ -19572,10 +19572,10 @@
         <v>679793.6</v>
       </c>
       <c r="J16">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K16">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L16">
         <v>479917.1</v>
@@ -19584,7 +19584,7 @@
         <v>787018</v>
       </c>
       <c r="N16">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O16">
         <v>210241.6</v>
@@ -19607,10 +19607,10 @@
         <v>129260</v>
       </c>
       <c r="F17">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G17">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H17">
         <v>382762.9</v>
@@ -19619,10 +19619,10 @@
         <v>679793.6</v>
       </c>
       <c r="J17">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K17">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L17">
         <v>479917.1</v>
@@ -19631,7 +19631,7 @@
         <v>787018</v>
       </c>
       <c r="N17">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O17">
         <v>205949.84</v>
@@ -19654,10 +19654,10 @@
         <v>127880</v>
       </c>
       <c r="F18">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H18">
         <v>382762.9</v>
@@ -19666,10 +19666,10 @@
         <v>679793.6</v>
       </c>
       <c r="J18">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K18">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L18">
         <v>479917.1</v>
@@ -19678,7 +19678,7 @@
         <v>787018</v>
       </c>
       <c r="N18">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O18">
         <v>201747.12</v>
@@ -19701,10 +19701,10 @@
         <v>126500</v>
       </c>
       <c r="F19">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H19">
         <v>382762.9</v>
@@ -19713,10 +19713,10 @@
         <v>679793.6</v>
       </c>
       <c r="J19">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K19">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L19">
         <v>479917.1</v>
@@ -19725,7 +19725,7 @@
         <v>787018</v>
       </c>
       <c r="N19">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O19">
         <v>197632.19</v>
@@ -19748,10 +19748,10 @@
         <v>125120</v>
       </c>
       <c r="F20">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H20">
         <v>382762.9</v>
@@ -19760,10 +19760,10 @@
         <v>679793.6</v>
       </c>
       <c r="J20">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K20">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L20">
         <v>479917.1</v>
@@ -19772,7 +19772,7 @@
         <v>787018</v>
       </c>
       <c r="N20">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O20">
         <v>193603.83</v>
@@ -19795,10 +19795,10 @@
         <v>123740</v>
       </c>
       <c r="F21">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G21">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H21">
         <v>382762.9</v>
@@ -19807,10 +19807,10 @@
         <v>679793.6</v>
       </c>
       <c r="J21">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K21">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L21">
         <v>479917.1</v>
@@ -19819,7 +19819,7 @@
         <v>787018</v>
       </c>
       <c r="N21">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O21">
         <v>189660.87</v>
@@ -19842,10 +19842,10 @@
         <v>122360</v>
       </c>
       <c r="F22">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H22">
         <v>382762.9</v>
@@ -19854,10 +19854,10 @@
         <v>679793.6</v>
       </c>
       <c r="J22">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K22">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L22">
         <v>479917.1</v>
@@ -19866,7 +19866,7 @@
         <v>787018</v>
       </c>
       <c r="N22">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O22">
         <v>185802.14</v>
@@ -19889,10 +19889,10 @@
         <v>120980</v>
       </c>
       <c r="F23">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H23">
         <v>382762.9</v>
@@ -19901,10 +19901,10 @@
         <v>679793.6</v>
       </c>
       <c r="J23">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K23">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L23">
         <v>479917.1</v>
@@ -19913,7 +19913,7 @@
         <v>787018</v>
       </c>
       <c r="N23">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O23">
         <v>182026.51</v>
@@ -19936,10 +19936,10 @@
         <v>119600</v>
       </c>
       <c r="F24">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G24">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H24">
         <v>382762.9</v>
@@ -19948,10 +19948,10 @@
         <v>679793.6</v>
       </c>
       <c r="J24">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K24">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L24">
         <v>479917.1</v>
@@ -19960,7 +19960,7 @@
         <v>787018</v>
       </c>
       <c r="N24">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O24">
         <v>178332.87</v>
@@ -19983,10 +19983,10 @@
         <v>118220</v>
       </c>
       <c r="F25">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G25">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H25">
         <v>382762.9</v>
@@ -19995,10 +19995,10 @@
         <v>679793.6</v>
       </c>
       <c r="J25">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K25">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L25">
         <v>479917.1</v>
@@ -20007,7 +20007,7 @@
         <v>787018</v>
       </c>
       <c r="N25">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O25">
         <v>174720.11</v>
@@ -20030,10 +20030,10 @@
         <v>116840</v>
       </c>
       <c r="F26">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H26">
         <v>382762.9</v>
@@ -20042,10 +20042,10 @@
         <v>679793.6</v>
       </c>
       <c r="J26">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K26">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L26">
         <v>479917.1</v>
@@ -20054,7 +20054,7 @@
         <v>787018</v>
       </c>
       <c r="N26">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O26">
         <v>171187.17</v>
@@ -20077,10 +20077,10 @@
         <v>115460</v>
       </c>
       <c r="F27">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H27">
         <v>382762.9</v>
@@ -20089,10 +20089,10 @@
         <v>679793.6</v>
       </c>
       <c r="J27">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K27">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L27">
         <v>479917.1</v>
@@ -20101,7 +20101,7 @@
         <v>787018</v>
       </c>
       <c r="N27">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O27">
         <v>167732.98000000001</v>
@@ -20124,10 +20124,10 @@
         <v>114080</v>
       </c>
       <c r="F28">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="H28">
         <v>382762.9</v>
@@ -20136,10 +20136,10 @@
         <v>679793.6</v>
       </c>
       <c r="J28">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="K28">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="L28">
         <v>479917.1</v>
@@ -20148,7 +20148,7 @@
         <v>787018</v>
       </c>
       <c r="N28">
-        <v>9999999</v>
+        <v>0</v>
       </c>
       <c r="O28">
         <v>164356.51999999999</v>

</xml_diff>

<commit_message>
removed LR10 from scenario generator and added a 4% LR to wind, whilst keeping 1.5% for SPV.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1387" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4F5CACF-96C4-4A92-BECE-A95E104C9789}"/>
+  <xr:revisionPtr revIDLastSave="1393" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9D21F25-9E48-4457-B384-0558FA00BE98}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6825" windowWidth="29040" windowHeight="17520" firstSheet="15" activeTab="21" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="4" activeTab="5" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -2785,6 +2785,26 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -2792,26 +2812,6 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -18955,10 +18955,10 @@
         <v>0</v>
       </c>
       <c r="H3">
-        <v>382762.9</v>
+        <v>367452.38400000002</v>
       </c>
       <c r="I3">
-        <v>679793.6</v>
+        <v>652601.85599999991</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -18967,10 +18967,10 @@
         <v>0</v>
       </c>
       <c r="L3">
-        <v>479917.1</v>
+        <v>460720.41599999997</v>
       </c>
       <c r="M3">
-        <v>787018</v>
+        <v>755537.28</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -19002,10 +19002,10 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>382762.9</v>
+        <v>352754.28863999998</v>
       </c>
       <c r="I4">
-        <v>679793.6</v>
+        <v>626497.78175999993</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -19014,10 +19014,10 @@
         <v>0</v>
       </c>
       <c r="L4">
-        <v>479917.1</v>
+        <v>442291.59935999993</v>
       </c>
       <c r="M4">
-        <v>787018</v>
+        <v>725315.78879999998</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -19049,10 +19049,10 @@
         <v>0</v>
       </c>
       <c r="H5">
-        <v>382762.9</v>
+        <v>338644.11709439999</v>
       </c>
       <c r="I5">
-        <v>679793.6</v>
+        <v>601437.87048959988</v>
       </c>
       <c r="J5">
         <v>0</v>
@@ -19061,10 +19061,10 @@
         <v>0</v>
       </c>
       <c r="L5">
-        <v>479917.1</v>
+        <v>424599.93538559991</v>
       </c>
       <c r="M5">
-        <v>787018</v>
+        <v>696303.15724799992</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -19096,10 +19096,10 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>382762.9</v>
+        <v>325098.35241062398</v>
       </c>
       <c r="I6">
-        <v>679793.6</v>
+        <v>577380.35567001591</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -19108,10 +19108,10 @@
         <v>0</v>
       </c>
       <c r="L6">
-        <v>479917.1</v>
+        <v>407615.93797017587</v>
       </c>
       <c r="M6">
-        <v>787018</v>
+        <v>668451.03095807985</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -19143,10 +19143,10 @@
         <v>0</v>
       </c>
       <c r="H7">
-        <v>382762.9</v>
+        <v>312094.41831419902</v>
       </c>
       <c r="I7">
-        <v>679793.6</v>
+        <v>554285.14144321531</v>
       </c>
       <c r="J7">
         <v>0</v>
@@ -19155,10 +19155,10 @@
         <v>0</v>
       </c>
       <c r="L7">
-        <v>479917.1</v>
+        <v>391311.30045136885</v>
       </c>
       <c r="M7">
-        <v>787018</v>
+        <v>641712.98971975665</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -19190,10 +19190,10 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>382762.9</v>
+        <v>299610.64158163103</v>
       </c>
       <c r="I8">
-        <v>679793.6</v>
+        <v>532113.73578548664</v>
       </c>
       <c r="J8">
         <v>0</v>
@@ -19202,10 +19202,10 @@
         <v>0</v>
       </c>
       <c r="L8">
-        <v>479917.1</v>
+        <v>375658.84843331407</v>
       </c>
       <c r="M8">
-        <v>787018</v>
+        <v>616044.47013096639</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -19237,10 +19237,10 @@
         <v>0</v>
       </c>
       <c r="H9">
-        <v>382762.9</v>
+        <v>287626.21591836581</v>
       </c>
       <c r="I9">
-        <v>679793.6</v>
+        <v>510829.18635406718</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -19249,10 +19249,10 @@
         <v>0</v>
       </c>
       <c r="L9">
-        <v>479917.1</v>
+        <v>360632.49449598149</v>
       </c>
       <c r="M9">
-        <v>787018</v>
+        <v>591402.69132572773</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -19284,10 +19284,10 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>382762.9</v>
+        <v>276121.16728163115</v>
       </c>
       <c r="I10">
-        <v>679793.6</v>
+        <v>490396.01889990445</v>
       </c>
       <c r="J10">
         <v>0</v>
@@ -19296,10 +19296,10 @@
         <v>0</v>
       </c>
       <c r="L10">
-        <v>479917.1</v>
+        <v>346207.1947161422</v>
       </c>
       <c r="M10">
-        <v>787018</v>
+        <v>567746.58367269859</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -19331,10 +19331,10 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>382762.9</v>
+        <v>265076.32059036591</v>
       </c>
       <c r="I11">
-        <v>679793.6</v>
+        <v>470780.17814390827</v>
       </c>
       <c r="J11">
         <v>0</v>
@@ -19343,10 +19343,10 @@
         <v>0</v>
       </c>
       <c r="L11">
-        <v>479917.1</v>
+        <v>332358.90692749649</v>
       </c>
       <c r="M11">
-        <v>787018</v>
+        <v>545036.72032579058</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -19378,10 +19378,10 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>382762.9</v>
+        <v>254473.26776675126</v>
       </c>
       <c r="I12">
-        <v>679793.6</v>
+        <v>451948.9710181519</v>
       </c>
       <c r="J12">
         <v>0</v>
@@ -19390,10 +19390,10 @@
         <v>0</v>
       </c>
       <c r="L12">
-        <v>479917.1</v>
+        <v>319064.55065039662</v>
       </c>
       <c r="M12">
-        <v>787018</v>
+        <v>523235.25151275896</v>
       </c>
       <c r="N12">
         <v>0</v>
@@ -19425,10 +19425,10 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>382762.9</v>
+        <v>244294.33705608119</v>
       </c>
       <c r="I13">
-        <v>679793.6</v>
+        <v>433871.01217742579</v>
       </c>
       <c r="J13">
         <v>0</v>
@@ -19437,10 +19437,10 @@
         <v>0</v>
       </c>
       <c r="L13">
-        <v>479917.1</v>
+        <v>306301.96862438077</v>
       </c>
       <c r="M13">
-        <v>787018</v>
+        <v>502305.84145224857</v>
       </c>
       <c r="N13">
         <v>0</v>
@@ -19472,10 +19472,10 @@
         <v>0</v>
       </c>
       <c r="H14">
-        <v>382762.9</v>
+        <v>234522.56357383792</v>
       </c>
       <c r="I14">
-        <v>679793.6</v>
+        <v>416516.17169032875</v>
       </c>
       <c r="J14">
         <v>0</v>
@@ -19484,10 +19484,10 @@
         <v>0</v>
       </c>
       <c r="L14">
-        <v>479917.1</v>
+        <v>294049.8898794055</v>
       </c>
       <c r="M14">
-        <v>787018</v>
+        <v>482213.60779415863</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -19519,10 +19519,10 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>382762.9</v>
+        <v>225141.6610308844</v>
       </c>
       <c r="I15">
-        <v>679793.6</v>
+        <v>399855.52482271555</v>
       </c>
       <c r="J15">
         <v>0</v>
@@ -19531,10 +19531,10 @@
         <v>0</v>
       </c>
       <c r="L15">
-        <v>479917.1</v>
+        <v>282287.89428422926</v>
       </c>
       <c r="M15">
-        <v>787018</v>
+        <v>462925.06348239229</v>
       </c>
       <c r="N15">
         <v>0</v>
@@ -19566,10 +19566,10 @@
         <v>0</v>
       </c>
       <c r="H16">
-        <v>382762.9</v>
+        <v>216135.99458964902</v>
       </c>
       <c r="I16">
-        <v>679793.6</v>
+        <v>383861.30382980692</v>
       </c>
       <c r="J16">
         <v>0</v>
@@ -19578,10 +19578,10 @@
         <v>0</v>
       </c>
       <c r="L16">
-        <v>479917.1</v>
+        <v>270996.3785128601</v>
       </c>
       <c r="M16">
-        <v>787018</v>
+        <v>444408.06094309659</v>
       </c>
       <c r="N16">
         <v>0</v>
@@ -19613,10 +19613,10 @@
         <v>0</v>
       </c>
       <c r="H17">
-        <v>382762.9</v>
+        <v>207490.55480606307</v>
       </c>
       <c r="I17">
-        <v>679793.6</v>
+        <v>368506.85167661461</v>
       </c>
       <c r="J17">
         <v>0</v>
@@ -19625,10 +19625,10 @@
         <v>0</v>
       </c>
       <c r="L17">
-        <v>479917.1</v>
+        <v>260156.52337234569</v>
       </c>
       <c r="M17">
-        <v>787018</v>
+        <v>426631.73850537272</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -19660,10 +19660,10 @@
         <v>0</v>
       </c>
       <c r="H18">
-        <v>382762.9</v>
+        <v>199190.93261382054</v>
       </c>
       <c r="I18">
-        <v>679793.6</v>
+        <v>353766.57760955003</v>
       </c>
       <c r="J18">
         <v>0</v>
@@ -19672,10 +19672,10 @@
         <v>0</v>
       </c>
       <c r="L18">
-        <v>479917.1</v>
+        <v>249750.26243745186</v>
       </c>
       <c r="M18">
-        <v>787018</v>
+        <v>409566.46896515781</v>
       </c>
       <c r="N18">
         <v>0</v>
@@ -19707,10 +19707,10 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>382762.9</v>
+        <v>191223.29530926771</v>
       </c>
       <c r="I19">
-        <v>679793.6</v>
+        <v>339615.91450516804</v>
       </c>
       <c r="J19">
         <v>0</v>
@@ -19719,10 +19719,10 @@
         <v>0</v>
       </c>
       <c r="L19">
-        <v>479917.1</v>
+        <v>239760.25193995377</v>
       </c>
       <c r="M19">
-        <v>787018</v>
+        <v>393183.81020655145</v>
       </c>
       <c r="N19">
         <v>0</v>
@@ -19754,10 +19754,10 @@
         <v>0</v>
       </c>
       <c r="H20">
-        <v>382762.9</v>
+        <v>183574.36349689699</v>
       </c>
       <c r="I20">
-        <v>679793.6</v>
+        <v>326031.27792496129</v>
       </c>
       <c r="J20">
         <v>0</v>
@@ -19766,10 +19766,10 @@
         <v>0</v>
       </c>
       <c r="L20">
-        <v>479917.1</v>
+        <v>230169.84186235562</v>
       </c>
       <c r="M20">
-        <v>787018</v>
+        <v>377456.45779828937</v>
       </c>
       <c r="N20">
         <v>0</v>
@@ -19801,10 +19801,10 @@
         <v>0</v>
       </c>
       <c r="H21">
-        <v>382762.9</v>
+        <v>176231.38895702109</v>
       </c>
       <c r="I21">
-        <v>679793.6</v>
+        <v>312990.02680796286</v>
       </c>
       <c r="J21">
         <v>0</v>
@@ -19813,10 +19813,10 @@
         <v>0</v>
       </c>
       <c r="L21">
-        <v>479917.1</v>
+        <v>220963.04818786139</v>
       </c>
       <c r="M21">
-        <v>787018</v>
+        <v>362358.1994863578</v>
       </c>
       <c r="N21">
         <v>0</v>
@@ -19848,10 +19848,10 @@
         <v>0</v>
       </c>
       <c r="H22">
-        <v>382762.9</v>
+        <v>169182.13339874023</v>
       </c>
       <c r="I22">
-        <v>679793.6</v>
+        <v>300470.42573564436</v>
       </c>
       <c r="J22">
         <v>0</v>
@@ -19860,10 +19860,10 @@
         <v>0</v>
       </c>
       <c r="L22">
-        <v>479917.1</v>
+        <v>212124.52626034693</v>
       </c>
       <c r="M22">
-        <v>787018</v>
+        <v>347863.8715069035</v>
       </c>
       <c r="N22">
         <v>0</v>
@@ -19895,10 +19895,10 @@
         <v>0</v>
       </c>
       <c r="H23">
-        <v>382762.9</v>
+        <v>162414.84806279061</v>
       </c>
       <c r="I23">
-        <v>679793.6</v>
+        <v>288451.6087062186</v>
       </c>
       <c r="J23">
         <v>0</v>
@@ -19907,10 +19907,10 @@
         <v>0</v>
       </c>
       <c r="L23">
-        <v>479917.1</v>
+        <v>203639.54520993304</v>
       </c>
       <c r="M23">
-        <v>787018</v>
+        <v>333949.31664662733</v>
       </c>
       <c r="N23">
         <v>0</v>
@@ -19942,10 +19942,10 @@
         <v>0</v>
       </c>
       <c r="H24">
-        <v>382762.9</v>
+        <v>155918.25414027899</v>
       </c>
       <c r="I24">
-        <v>679793.6</v>
+        <v>276913.54435796983</v>
       </c>
       <c r="J24">
         <v>0</v>
@@ -19954,10 +19954,10 @@
         <v>0</v>
       </c>
       <c r="L24">
-        <v>479917.1</v>
+        <v>195493.9634015357</v>
       </c>
       <c r="M24">
-        <v>787018</v>
+        <v>320591.34398076223</v>
       </c>
       <c r="N24">
         <v>0</v>
@@ -19989,10 +19989,10 @@
         <v>0</v>
       </c>
       <c r="H25">
-        <v>382762.9</v>
+        <v>149681.52397466783</v>
       </c>
       <c r="I25">
-        <v>679793.6</v>
+        <v>265837.00258365105</v>
       </c>
       <c r="J25">
         <v>0</v>
@@ -20001,10 +20001,10 @@
         <v>0</v>
       </c>
       <c r="L25">
-        <v>479917.1</v>
+        <v>187674.20486547425</v>
       </c>
       <c r="M25">
-        <v>787018</v>
+        <v>307767.69022153172</v>
       </c>
       <c r="N25">
         <v>0</v>
@@ -20036,10 +20036,10 @@
         <v>0</v>
       </c>
       <c r="H26">
-        <v>382762.9</v>
+        <v>143694.26301568112</v>
       </c>
       <c r="I26">
-        <v>679793.6</v>
+        <v>255203.52248030499</v>
       </c>
       <c r="J26">
         <v>0</v>
@@ -20048,10 +20048,10 @@
         <v>0</v>
       </c>
       <c r="L26">
-        <v>479917.1</v>
+        <v>180167.23667085529</v>
       </c>
       <c r="M26">
-        <v>787018</v>
+        <v>295456.98261267046</v>
       </c>
       <c r="N26">
         <v>0</v>
@@ -20083,10 +20083,10 @@
         <v>0</v>
       </c>
       <c r="H27">
-        <v>382762.9</v>
+        <v>137946.49249505388</v>
       </c>
       <c r="I27">
-        <v>679793.6</v>
+        <v>244995.38158109278</v>
       </c>
       <c r="J27">
         <v>0</v>
@@ -20095,10 +20095,10 @@
         <v>0</v>
       </c>
       <c r="L27">
-        <v>479917.1</v>
+        <v>172960.54720402107</v>
       </c>
       <c r="M27">
-        <v>787018</v>
+        <v>283638.70330816362</v>
       </c>
       <c r="N27">
         <v>0</v>
@@ -20130,10 +20130,10 @@
         <v>0</v>
       </c>
       <c r="H28">
-        <v>382762.9</v>
+        <v>132428.63279525173</v>
       </c>
       <c r="I28">
-        <v>679793.6</v>
+        <v>235195.56631784906</v>
       </c>
       <c r="J28">
         <v>0</v>
@@ -20142,10 +20142,10 @@
         <v>0</v>
       </c>
       <c r="L28">
-        <v>479917.1</v>
+        <v>166042.12531586023</v>
       </c>
       <c r="M28">
-        <v>787018</v>
+        <v>272293.15517583705</v>
       </c>
       <c r="N28">
         <v>0</v>

</xml_diff>

<commit_message>
Revised Recycling Cost for SPV
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1393" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9D21F25-9E48-4457-B384-0558FA00BE98}"/>
+  <xr:revisionPtr revIDLastSave="1395" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{333336BF-3C35-48B9-9855-A6608C6399A2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="4" activeTab="5" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="8" activeTab="12" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="199">
   <si>
     <t>Value</t>
   </si>
@@ -399,18 +399,6 @@
   </si>
   <si>
     <t>opex_fixed</t>
-  </si>
-  <si>
-    <t>0.98</t>
-  </si>
-  <si>
-    <t>0.994</t>
-  </si>
-  <si>
-    <t>0.97</t>
-  </si>
-  <si>
-    <t>0.94</t>
   </si>
   <si>
     <t>CellBatt</t>
@@ -1020,10 +1008,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -2785,26 +2769,6 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -2812,6 +2776,26 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2951,7 +2935,7 @@
         <v>76</v>
       </c>
       <c r="C6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -2977,7 +2961,7 @@
         <v>76</v>
       </c>
       <c r="C7" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -3003,7 +2987,7 @@
         <v>76</v>
       </c>
       <c r="C8" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -3029,7 +3013,7 @@
         <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -3055,7 +3039,7 @@
         <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -3081,7 +3065,7 @@
         <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -3104,7 +3088,7 @@
         <v>77</v>
       </c>
       <c r="C12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -3127,7 +3111,7 @@
         <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -3150,7 +3134,7 @@
         <v>88</v>
       </c>
       <c r="C14" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -3235,7 +3219,7 @@
         <v>87</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D2" s="12">
         <v>11.080597014925374</v>
@@ -3243,8 +3227,8 @@
       <c r="E2" s="12">
         <v>11.080597014925374</v>
       </c>
-      <c r="F2" s="12" t="s">
-        <v>114</v>
+      <c r="F2">
+        <v>0.99399999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -3255,7 +3239,7 @@
         <v>87</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D3" s="12">
         <v>46.4</v>
@@ -3263,8 +3247,8 @@
       <c r="E3" s="12">
         <v>46.4</v>
       </c>
-      <c r="F3" s="12" t="s">
-        <v>113</v>
+      <c r="F3">
+        <v>0.92100000000000004</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -3275,7 +3259,7 @@
         <v>87</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D4" s="12">
         <v>7.6179104477611936</v>
@@ -3283,8 +3267,8 @@
       <c r="E4" s="12">
         <v>7.6179104477611936</v>
       </c>
-      <c r="F4" s="12" t="s">
-        <v>85</v>
+      <c r="F4">
+        <v>0.27400000000000002</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -3295,7 +3279,7 @@
         <v>87</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D5" s="12">
         <v>0.62328358208955215</v>
@@ -3303,8 +3287,8 @@
       <c r="E5" s="12">
         <v>0.62328358208955215</v>
       </c>
-      <c r="F5" s="12" t="s">
-        <v>115</v>
+      <c r="F5">
+        <v>0.97</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -3315,7 +3299,7 @@
         <v>86</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D6" s="12">
         <v>2.0776119402985072E-2</v>
@@ -3323,8 +3307,8 @@
       <c r="E6" s="12">
         <v>2.0776119402985072E-2</v>
       </c>
-      <c r="F6" s="12" t="s">
-        <v>116</v>
+      <c r="F6">
+        <v>0.68100000000000005</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -3335,7 +3319,7 @@
         <v>108</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D7" s="12">
         <v>3.047164179104477</v>
@@ -3343,8 +3327,8 @@
       <c r="E7" s="12">
         <v>3.047164179104477</v>
       </c>
-      <c r="F7" s="12" t="s">
-        <v>115</v>
+      <c r="F7">
+        <v>0.88900000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -3355,7 +3339,7 @@
         <v>86</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D8" s="12">
         <v>0.20776119402985074</v>
@@ -3363,8 +3347,8 @@
       <c r="E8" s="12">
         <v>0.20776119402985074</v>
       </c>
-      <c r="F8" s="12" t="s">
-        <v>114</v>
+      <c r="F8">
+        <v>0.1</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -3372,10 +3356,10 @@
         <v>76</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D9" s="12">
         <v>15</v>
@@ -3392,10 +3376,10 @@
         <v>76</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D10" s="12">
         <v>180</v>
@@ -3412,10 +3396,10 @@
         <v>76</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D11" s="12">
         <v>0.80645121600000003</v>
@@ -3432,10 +3416,10 @@
         <v>76</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D12" s="12">
         <v>2.4417760000000005E-3</v>
@@ -3452,10 +3436,10 @@
         <v>76</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D13" s="12">
         <v>0.99598527400000014</v>
@@ -3472,10 +3456,10 @@
         <v>76</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D14" s="12">
         <v>1.8875200000000002E-3</v>
@@ -3492,10 +3476,10 @@
         <v>76</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D15" s="12">
         <v>4.4819000000000006E-5</v>
@@ -3512,10 +3496,10 @@
         <v>76</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D16" s="12">
         <v>4.6005630000000002E-3</v>
@@ -3532,10 +3516,10 @@
         <v>76</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D17" s="12">
         <v>9.0565300000000008E-4</v>
@@ -3552,10 +3536,10 @@
         <v>76</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D18" s="12">
         <v>1.9774658839999999</v>
@@ -3572,10 +3556,10 @@
         <v>76</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D19" s="12">
         <v>3.9663748000000006E-2</v>
@@ -3592,10 +3576,10 @@
         <v>76</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D20" s="12">
         <v>2.1210528159999997</v>
@@ -3612,10 +3596,10 @@
         <v>76</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D21" s="12">
         <v>3.0464200000000004E-4</v>
@@ -3632,10 +3616,10 @@
         <v>76</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D22" s="12">
         <v>5.3289600000000004E-4</v>
@@ -3652,10 +3636,10 @@
         <v>76</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D23" s="12">
         <v>2.3000000000000001E-8</v>
@@ -3672,10 +3656,10 @@
         <v>76</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D24" s="12">
         <v>5.0735241E-2</v>
@@ -3692,10 +3676,10 @@
         <v>76</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D25" s="12">
         <v>1.5200000000000001E-7</v>
@@ -3712,10 +3696,10 @@
         <v>77</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D26" s="12">
         <v>30</v>
@@ -3732,10 +3716,10 @@
         <v>77</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D27" s="12">
         <v>250</v>
@@ -3752,10 +3736,10 @@
         <v>77</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D28" s="12">
         <v>0.76185761500000004</v>
@@ -3772,10 +3756,10 @@
         <v>77</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D29" s="12">
         <v>2.0542469999999995E-3</v>
@@ -3792,10 +3776,10 @@
         <v>77</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D30" s="12">
         <v>1.3319019999999998E-3</v>
@@ -3812,10 +3796,10 @@
         <v>77</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D31" s="12">
         <v>1.5534533760000002</v>
@@ -3832,10 +3816,10 @@
         <v>77</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D32" s="12">
         <v>6.5629390000000003E-3</v>
@@ -3852,10 +3836,10 @@
         <v>77</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D33" s="12">
         <v>1.592E-5</v>
@@ -3872,10 +3856,10 @@
         <v>77</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D34" s="12">
         <v>6.3938059999999993E-3</v>
@@ -3892,10 +3876,10 @@
         <v>77</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D35" s="12">
         <v>1.2656820000000002E-3</v>
@@ -3912,10 +3896,10 @@
         <v>77</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D36" s="12">
         <v>1.0573537260000001</v>
@@ -3932,10 +3916,10 @@
         <v>77</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D37" s="12">
         <v>3.7349899999999996E-4</v>
@@ -3952,10 +3936,10 @@
         <v>77</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D38" s="12">
         <v>0.10560918700000001</v>
@@ -3972,10 +3956,10 @@
         <v>77</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D39" s="12">
         <v>0.86241605300000002</v>
@@ -3992,10 +3976,10 @@
         <v>77</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D40" s="12">
         <v>1.59808E-4</v>
@@ -4012,10 +3996,10 @@
         <v>77</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D41" s="12">
         <v>4.3179209999999996E-2</v>
@@ -4032,10 +4016,10 @@
         <v>77</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D42" s="12">
         <v>3.7350900000000006E-4</v>
@@ -4052,10 +4036,10 @@
         <v>77</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D43" s="12">
         <v>2.6648077999999999E-2</v>
@@ -4072,10 +4056,10 @@
         <v>77</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D44" s="12">
         <v>4.3999999999999997E-8</v>
@@ -4092,10 +4076,10 @@
         <v>88</v>
       </c>
       <c r="B45" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D45">
         <v>0</v>
@@ -4112,10 +4096,10 @@
         <v>88</v>
       </c>
       <c r="B46" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C46" s="18" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D46">
         <v>0</v>
@@ -4147,31 +4131,31 @@
         <v>82</v>
       </c>
       <c r="C1" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="D1" t="s">
         <v>112</v>
       </c>
       <c r="E1" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1" t="s">
+        <v>191</v>
+      </c>
+      <c r="G1" t="s">
+        <v>195</v>
+      </c>
+      <c r="H1" t="s">
+        <v>196</v>
+      </c>
+      <c r="I1" t="s">
+        <v>192</v>
+      </c>
+      <c r="J1" t="s">
+        <v>197</v>
+      </c>
+      <c r="K1" t="s">
         <v>198</v>
-      </c>
-      <c r="F1" t="s">
-        <v>195</v>
-      </c>
-      <c r="G1" t="s">
-        <v>199</v>
-      </c>
-      <c r="H1" t="s">
-        <v>200</v>
-      </c>
-      <c r="I1" t="s">
-        <v>196</v>
-      </c>
-      <c r="J1" t="s">
-        <v>201</v>
-      </c>
-      <c r="K1" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -4252,13 +4236,13 @@
         <v>75</v>
       </c>
       <c r="C4">
-        <v>494.690808</v>
+        <v>365.87143333333336</v>
       </c>
       <c r="D4">
-        <v>1225.6664426666666</v>
+        <v>580.25940740740748</v>
       </c>
       <c r="E4">
-        <v>1225.44</v>
+        <v>165.14292592592594</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -4331,36 +4315,36 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C1" t="s">
+        <v>183</v>
+      </c>
+      <c r="D1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E1" t="s">
         <v>185</v>
       </c>
-      <c r="B1" t="s">
+      <c r="F1" t="s">
         <v>186</v>
       </c>
-      <c r="C1" t="s">
+      <c r="G1" t="s">
         <v>187</v>
       </c>
-      <c r="D1" t="s">
+      <c r="H1" t="s">
         <v>188</v>
       </c>
-      <c r="E1" t="s">
+      <c r="I1" t="s">
         <v>189</v>
-      </c>
-      <c r="F1" t="s">
-        <v>190</v>
-      </c>
-      <c r="G1" t="s">
-        <v>191</v>
-      </c>
-      <c r="H1" t="s">
-        <v>192</v>
-      </c>
-      <c r="I1" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B2">
         <v>227523.06210000001</v>
@@ -4391,7 +4375,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B3">
         <v>1090137.72</v>
@@ -4422,7 +4406,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B4">
         <v>189432.22750000001</v>
@@ -4453,7 +4437,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B5">
         <v>94712.809810000006</v>
@@ -4484,7 +4468,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B6">
         <v>541.22898280000004</v>
@@ -4515,7 +4499,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B7">
         <v>58452.73014</v>
@@ -4546,7 +4530,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B8">
         <v>143</v>
@@ -4577,7 +4561,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B9">
         <v>57.291095110000001</v>
@@ -4608,7 +4592,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B10">
         <v>3.2587681910000001</v>
@@ -4639,7 +4623,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B11">
         <v>1068</v>
@@ -4670,7 +4654,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B12">
         <v>133</v>
@@ -4701,7 +4685,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B13">
         <v>9206.9589369999994</v>
@@ -4732,7 +4716,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B14">
         <v>512.35706370000003</v>
@@ -4763,7 +4747,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B15">
         <v>3774.5654399999999</v>
@@ -4794,7 +4778,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B16">
         <v>999999</v>
@@ -4825,7 +4809,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B17">
         <v>83.438261490000002</v>
@@ -4856,7 +4840,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B18">
         <v>19.865756780000002</v>
@@ -4887,7 +4871,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B19">
         <v>999999</v>
@@ -4918,7 +4902,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B20">
         <v>999999</v>
@@ -4949,7 +4933,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B21">
         <v>13.73426465</v>
@@ -4980,7 +4964,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B22">
         <v>1038.9856569999999</v>
@@ -5011,7 +4995,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B23">
         <v>999999</v>
@@ -5042,7 +5026,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B24">
         <v>999999</v>
@@ -5073,7 +5057,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B25">
         <v>999999</v>
@@ -5104,7 +5088,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B26">
         <v>999999</v>
@@ -5148,79 +5132,79 @@
         <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E1" t="s">
+        <v>156</v>
+      </c>
+      <c r="F1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G1" t="s">
+        <v>176</v>
+      </c>
+      <c r="H1" t="s">
+        <v>153</v>
+      </c>
+      <c r="I1" t="s">
+        <v>154</v>
+      </c>
+      <c r="J1" t="s">
+        <v>155</v>
+      </c>
+      <c r="K1" t="s">
+        <v>157</v>
+      </c>
+      <c r="L1" t="s">
+        <v>158</v>
+      </c>
+      <c r="M1" t="s">
+        <v>159</v>
+      </c>
+      <c r="N1" t="s">
         <v>160</v>
       </c>
-      <c r="F1" t="s">
-        <v>179</v>
-      </c>
-      <c r="G1" t="s">
-        <v>180</v>
-      </c>
-      <c r="H1" t="s">
-        <v>157</v>
-      </c>
-      <c r="I1" t="s">
-        <v>158</v>
-      </c>
-      <c r="J1" t="s">
-        <v>159</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="O1" t="s">
         <v>161</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>162</v>
       </c>
-      <c r="M1" t="s">
+      <c r="Q1" t="s">
         <v>163</v>
       </c>
-      <c r="N1" t="s">
+      <c r="R1" t="s">
         <v>164</v>
       </c>
-      <c r="O1" t="s">
+      <c r="S1" t="s">
         <v>165</v>
       </c>
-      <c r="P1" t="s">
+      <c r="T1" t="s">
         <v>166</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="U1" t="s">
         <v>167</v>
       </c>
-      <c r="R1" t="s">
+      <c r="V1" t="s">
         <v>168</v>
       </c>
-      <c r="S1" t="s">
+      <c r="W1" t="s">
         <v>169</v>
       </c>
-      <c r="T1" t="s">
+      <c r="X1" t="s">
         <v>170</v>
       </c>
-      <c r="U1" t="s">
+      <c r="Y1" t="s">
         <v>171</v>
       </c>
-      <c r="V1" t="s">
+      <c r="Z1" t="s">
         <v>172</v>
-      </c>
-      <c r="W1" t="s">
-        <v>173</v>
-      </c>
-      <c r="X1" t="s">
-        <v>174</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>175</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
@@ -7398,79 +7382,79 @@
         <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E1" t="s">
+        <v>156</v>
+      </c>
+      <c r="F1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G1" t="s">
+        <v>176</v>
+      </c>
+      <c r="H1" t="s">
+        <v>153</v>
+      </c>
+      <c r="I1" t="s">
+        <v>154</v>
+      </c>
+      <c r="J1" t="s">
+        <v>155</v>
+      </c>
+      <c r="K1" t="s">
+        <v>157</v>
+      </c>
+      <c r="L1" t="s">
+        <v>158</v>
+      </c>
+      <c r="M1" t="s">
+        <v>159</v>
+      </c>
+      <c r="N1" t="s">
         <v>160</v>
       </c>
-      <c r="F1" t="s">
-        <v>179</v>
-      </c>
-      <c r="G1" t="s">
-        <v>180</v>
-      </c>
-      <c r="H1" t="s">
-        <v>157</v>
-      </c>
-      <c r="I1" t="s">
-        <v>158</v>
-      </c>
-      <c r="J1" t="s">
-        <v>159</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="O1" t="s">
         <v>161</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>162</v>
       </c>
-      <c r="M1" t="s">
+      <c r="Q1" t="s">
         <v>163</v>
       </c>
-      <c r="N1" t="s">
+      <c r="R1" t="s">
         <v>164</v>
       </c>
-      <c r="O1" t="s">
+      <c r="S1" t="s">
         <v>165</v>
       </c>
-      <c r="P1" t="s">
+      <c r="T1" t="s">
         <v>166</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="U1" t="s">
         <v>167</v>
       </c>
-      <c r="R1" t="s">
+      <c r="V1" t="s">
         <v>168</v>
       </c>
-      <c r="S1" t="s">
+      <c r="W1" t="s">
         <v>169</v>
       </c>
-      <c r="T1" t="s">
+      <c r="X1" t="s">
         <v>170</v>
       </c>
-      <c r="U1" t="s">
+      <c r="Y1" t="s">
         <v>171</v>
       </c>
-      <c r="V1" t="s">
+      <c r="Z1" t="s">
         <v>172</v>
-      </c>
-      <c r="W1" t="s">
-        <v>173</v>
-      </c>
-      <c r="X1" t="s">
-        <v>174</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>175</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
@@ -9648,79 +9632,79 @@
         <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E1" t="s">
+        <v>156</v>
+      </c>
+      <c r="F1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G1" t="s">
+        <v>176</v>
+      </c>
+      <c r="H1" t="s">
+        <v>153</v>
+      </c>
+      <c r="I1" t="s">
+        <v>154</v>
+      </c>
+      <c r="J1" t="s">
+        <v>155</v>
+      </c>
+      <c r="K1" t="s">
+        <v>157</v>
+      </c>
+      <c r="L1" t="s">
+        <v>158</v>
+      </c>
+      <c r="M1" t="s">
+        <v>159</v>
+      </c>
+      <c r="N1" t="s">
         <v>160</v>
       </c>
-      <c r="F1" t="s">
-        <v>179</v>
-      </c>
-      <c r="G1" t="s">
-        <v>180</v>
-      </c>
-      <c r="H1" t="s">
-        <v>157</v>
-      </c>
-      <c r="I1" t="s">
-        <v>158</v>
-      </c>
-      <c r="J1" t="s">
-        <v>159</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="O1" t="s">
         <v>161</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>162</v>
       </c>
-      <c r="M1" t="s">
+      <c r="Q1" t="s">
         <v>163</v>
       </c>
-      <c r="N1" t="s">
+      <c r="R1" t="s">
         <v>164</v>
       </c>
-      <c r="O1" t="s">
+      <c r="S1" t="s">
         <v>165</v>
       </c>
-      <c r="P1" t="s">
+      <c r="T1" t="s">
         <v>166</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="U1" t="s">
         <v>167</v>
       </c>
-      <c r="R1" t="s">
+      <c r="V1" t="s">
         <v>168</v>
       </c>
-      <c r="S1" t="s">
+      <c r="W1" t="s">
         <v>169</v>
       </c>
-      <c r="T1" t="s">
+      <c r="X1" t="s">
         <v>170</v>
       </c>
-      <c r="U1" t="s">
+      <c r="Y1" t="s">
         <v>171</v>
       </c>
-      <c r="V1" t="s">
+      <c r="Z1" t="s">
         <v>172</v>
-      </c>
-      <c r="W1" t="s">
-        <v>173</v>
-      </c>
-      <c r="X1" t="s">
-        <v>174</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>175</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
@@ -11898,79 +11882,79 @@
         <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E1" t="s">
+        <v>156</v>
+      </c>
+      <c r="F1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G1" t="s">
+        <v>176</v>
+      </c>
+      <c r="H1" t="s">
+        <v>153</v>
+      </c>
+      <c r="I1" t="s">
+        <v>154</v>
+      </c>
+      <c r="J1" t="s">
+        <v>155</v>
+      </c>
+      <c r="K1" t="s">
+        <v>157</v>
+      </c>
+      <c r="L1" t="s">
+        <v>158</v>
+      </c>
+      <c r="M1" t="s">
+        <v>159</v>
+      </c>
+      <c r="N1" t="s">
         <v>160</v>
       </c>
-      <c r="F1" t="s">
-        <v>179</v>
-      </c>
-      <c r="G1" t="s">
-        <v>180</v>
-      </c>
-      <c r="H1" t="s">
-        <v>157</v>
-      </c>
-      <c r="I1" t="s">
-        <v>158</v>
-      </c>
-      <c r="J1" t="s">
-        <v>159</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="O1" t="s">
         <v>161</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>162</v>
       </c>
-      <c r="M1" t="s">
+      <c r="Q1" t="s">
         <v>163</v>
       </c>
-      <c r="N1" t="s">
+      <c r="R1" t="s">
         <v>164</v>
       </c>
-      <c r="O1" t="s">
+      <c r="S1" t="s">
         <v>165</v>
       </c>
-      <c r="P1" t="s">
+      <c r="T1" t="s">
         <v>166</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="U1" t="s">
         <v>167</v>
       </c>
-      <c r="R1" t="s">
+      <c r="V1" t="s">
         <v>168</v>
       </c>
-      <c r="S1" t="s">
+      <c r="W1" t="s">
         <v>169</v>
       </c>
-      <c r="T1" t="s">
+      <c r="X1" t="s">
         <v>170</v>
       </c>
-      <c r="U1" t="s">
+      <c r="Y1" t="s">
         <v>171</v>
       </c>
-      <c r="V1" t="s">
+      <c r="Z1" t="s">
         <v>172</v>
-      </c>
-      <c r="W1" t="s">
-        <v>173</v>
-      </c>
-      <c r="X1" t="s">
-        <v>174</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>175</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
@@ -14148,79 +14132,79 @@
         <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E1" t="s">
+        <v>156</v>
+      </c>
+      <c r="F1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G1" t="s">
+        <v>176</v>
+      </c>
+      <c r="H1" t="s">
+        <v>153</v>
+      </c>
+      <c r="I1" t="s">
+        <v>154</v>
+      </c>
+      <c r="J1" t="s">
+        <v>155</v>
+      </c>
+      <c r="K1" t="s">
+        <v>157</v>
+      </c>
+      <c r="L1" t="s">
+        <v>158</v>
+      </c>
+      <c r="M1" t="s">
+        <v>159</v>
+      </c>
+      <c r="N1" t="s">
         <v>160</v>
       </c>
-      <c r="F1" t="s">
-        <v>179</v>
-      </c>
-      <c r="G1" t="s">
-        <v>180</v>
-      </c>
-      <c r="H1" t="s">
-        <v>157</v>
-      </c>
-      <c r="I1" t="s">
-        <v>158</v>
-      </c>
-      <c r="J1" t="s">
-        <v>159</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="O1" t="s">
         <v>161</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>162</v>
       </c>
-      <c r="M1" t="s">
+      <c r="Q1" t="s">
         <v>163</v>
       </c>
-      <c r="N1" t="s">
+      <c r="R1" t="s">
         <v>164</v>
       </c>
-      <c r="O1" t="s">
+      <c r="S1" t="s">
         <v>165</v>
       </c>
-      <c r="P1" t="s">
+      <c r="T1" t="s">
         <v>166</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="U1" t="s">
         <v>167</v>
       </c>
-      <c r="R1" t="s">
+      <c r="V1" t="s">
         <v>168</v>
       </c>
-      <c r="S1" t="s">
+      <c r="W1" t="s">
         <v>169</v>
       </c>
-      <c r="T1" t="s">
+      <c r="X1" t="s">
         <v>170</v>
       </c>
-      <c r="U1" t="s">
+      <c r="Y1" t="s">
         <v>171</v>
       </c>
-      <c r="V1" t="s">
-        <v>172</v>
-      </c>
-      <c r="W1" t="s">
-        <v>173</v>
-      </c>
-      <c r="X1" t="s">
-        <v>174</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>175</v>
-      </c>
       <c r="Z1" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
@@ -18319,7 +18303,7 @@
         <v>88</v>
       </c>
       <c r="D5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E5" t="s">
         <v>92</v>
@@ -18330,13 +18314,13 @@
         <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C6" t="s">
         <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E6" t="s">
         <v>92</v>
@@ -18347,13 +18331,13 @@
         <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C7" t="s">
         <v>76</v>
       </c>
       <c r="D7" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E7" t="s">
         <v>92</v>
@@ -18364,13 +18348,13 @@
         <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C8" t="s">
         <v>76</v>
       </c>
       <c r="D8" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E8" t="s">
         <v>92</v>
@@ -18381,13 +18365,13 @@
         <v>77</v>
       </c>
       <c r="B9" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C9" t="s">
         <v>77</v>
       </c>
       <c r="D9" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E9" t="s">
         <v>92</v>
@@ -18398,13 +18382,13 @@
         <v>77</v>
       </c>
       <c r="B10" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C10" t="s">
         <v>77</v>
       </c>
       <c r="D10" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E10" t="s">
         <v>92</v>
@@ -18415,13 +18399,13 @@
         <v>77</v>
       </c>
       <c r="B11" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C11" t="s">
         <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="E11" t="s">
         <v>92</v>
@@ -18460,7 +18444,7 @@
         <v>112</v>
       </c>
       <c r="H1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -18578,7 +18562,7 @@
         <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E6" s="12">
         <v>73600</v>
@@ -18604,7 +18588,7 @@
         <v>76</v>
       </c>
       <c r="D7" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E7" s="12">
         <v>82800</v>
@@ -18630,7 +18614,7 @@
         <v>76</v>
       </c>
       <c r="D8" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E8" s="12">
         <v>276000</v>
@@ -18656,7 +18640,7 @@
         <v>76</v>
       </c>
       <c r="D9" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
@@ -18682,7 +18666,7 @@
         <v>77</v>
       </c>
       <c r="D10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E10" s="12">
         <v>165600</v>
@@ -18708,7 +18692,7 @@
         <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E11" s="12">
         <v>202400</v>
@@ -18734,7 +18718,7 @@
         <v>77</v>
       </c>
       <c r="D12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="E12" s="12">
         <v>202400</v>
@@ -18760,7 +18744,7 @@
         <v>77</v>
       </c>
       <c r="D13" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E13" s="12">
         <v>1</v>
@@ -18786,7 +18770,7 @@
         <v>88</v>
       </c>
       <c r="D14" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -18855,31 +18839,31 @@
         <v>107</v>
       </c>
       <c r="F1" t="s">
+        <v>128</v>
+      </c>
+      <c r="G1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H1" t="s">
+        <v>130</v>
+      </c>
+      <c r="I1" t="s">
+        <v>131</v>
+      </c>
+      <c r="J1" t="s">
         <v>132</v>
       </c>
-      <c r="G1" t="s">
+      <c r="K1" t="s">
         <v>133</v>
       </c>
-      <c r="H1" t="s">
+      <c r="L1" t="s">
         <v>134</v>
       </c>
-      <c r="I1" t="s">
+      <c r="M1" t="s">
         <v>135</v>
       </c>
-      <c r="J1" t="s">
-        <v>136</v>
-      </c>
-      <c r="K1" t="s">
-        <v>137</v>
-      </c>
-      <c r="L1" t="s">
-        <v>138</v>
-      </c>
-      <c r="M1" t="s">
-        <v>139</v>
-      </c>
       <c r="N1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="O1" t="s">
         <v>110</v>
@@ -27243,7 +27227,7 @@
         <v>77</v>
       </c>
       <c r="H1" s="23" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
update github repo with current problem of very few sPV installed due tu silicon bottlekneck
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1395" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{333336BF-3C35-48B9-9855-A6608C6399A2}"/>
+  <xr:revisionPtr revIDLastSave="1397" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC22F778-984B-4F26-96AC-1AFE0017F743}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="8" activeTab="12" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="38280" yWindow="0" windowWidth="38640" windowHeight="21120" firstSheet="8" activeTab="11" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>

</xml_diff>

<commit_message>
feat(model): integrate DEA BOS timeseries, tech-specific lifetimes and weighted VOM
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="11_9CEC12624582B70A48B9777787B9EB57C6EAF28B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2AF5255B-E734-4E6C-8683-7012B7211158}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_DC7891F35646FCA8E8287266FD6BDB1CEF623CDD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA15C6BA-FE05-4060-A44D-47FF38828687}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="15" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="1" r:id="rId1"/>
@@ -58,6 +58,174 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="208">
+  <si>
+    <t>Stf</t>
+  </si>
+  <si>
+    <t>solarPV_Polysilicon</t>
+  </si>
+  <si>
+    <t>solarPV_Wafer</t>
+  </si>
+  <si>
+    <t>solarPV_Cell</t>
+  </si>
+  <si>
+    <t>solarPV_Module</t>
+  </si>
+  <si>
+    <t>windon_BladeOn</t>
+  </si>
+  <si>
+    <t>windon_TowerOn</t>
+  </si>
+  <si>
+    <t>windon_NacelleOn</t>
+  </si>
+  <si>
+    <t>windon_AssemblyOn</t>
+  </si>
+  <si>
+    <t>windoff_BladeOff</t>
+  </si>
+  <si>
+    <t>windoff_TowerOff</t>
+  </si>
+  <si>
+    <t>windoff_NacelleOff</t>
+  </si>
+  <si>
+    <t>windoff_AssemblyOff</t>
+  </si>
+  <si>
+    <t>Batteries_CellBatt</t>
+  </si>
+  <si>
+    <t>Batteries_Assembly</t>
+  </si>
+  <si>
+    <t>capex_solarPV_bos</t>
+  </si>
+  <si>
+    <t>capex_windon_bos</t>
+  </si>
+  <si>
+    <t>capex_windoff_bos</t>
+  </si>
+  <si>
+    <t>opexf_solarPV_bos</t>
+  </si>
+  <si>
+    <t>opexf_windon_bos</t>
+  </si>
+  <si>
+    <t>opexf_windoff_bos</t>
+  </si>
+  <si>
+    <t>opexv_solarPV_bos</t>
+  </si>
+  <si>
+    <t>opexv_windon_bos</t>
+  </si>
+  <si>
+    <t>opexv_windoff_bos</t>
+  </si>
+  <si>
+    <t>Param</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Start Year y0</t>
+  </si>
+  <si>
+    <t>End Year yn</t>
+  </si>
+  <si>
+    <t>hours per year</t>
+  </si>
+  <si>
+    <t>import_EU27_solarPV</t>
+  </si>
+  <si>
+    <t>manufacturing_EU27_solarPV</t>
+  </si>
+  <si>
+    <t>remanufacturing_EU27_solarPV</t>
+  </si>
+  <si>
+    <t>recycling_EU27_solarPV</t>
+  </si>
+  <si>
+    <t>oandm_EU27_solarPV</t>
+  </si>
+  <si>
+    <t>import_EU27_windoff</t>
+  </si>
+  <si>
+    <t>manufacturing_EU27_windoff</t>
+  </si>
+  <si>
+    <t>remanufacturing_EU27_windoff</t>
+  </si>
+  <si>
+    <t>recycling_EU27_windoff</t>
+  </si>
+  <si>
+    <t>oandm_EU27_windoff</t>
+  </si>
+  <si>
+    <t>import_EU27_windon</t>
+  </si>
+  <si>
+    <t>manufacturing_EU27_windon</t>
+  </si>
+  <si>
+    <t>remanufacturing_EU27_windon</t>
+  </si>
+  <si>
+    <t>recycling_EU27_windon</t>
+  </si>
+  <si>
+    <t>oandm_EU27_windon</t>
+  </si>
+  <si>
+    <t>import_EU27_Batteries</t>
+  </si>
+  <si>
+    <t>manufacturing_EU27_Batteries</t>
+  </si>
+  <si>
+    <t>remanufacturing_EU27_Batteries</t>
+  </si>
+  <si>
+    <t>recycling_EU27_Batteries</t>
+  </si>
+  <si>
+    <t>oandm_EU27_Batteries</t>
+  </si>
+  <si>
+    <t>Locations:</t>
+  </si>
+  <si>
+    <t>EU27</t>
+  </si>
+  <si>
+    <t>timestep</t>
+  </si>
+  <si>
+    <t>EU27_solarPV</t>
+  </si>
+  <si>
+    <t>EU27_windoff</t>
+  </si>
+  <si>
+    <t>EU27_windon</t>
+  </si>
+  <si>
+    <t>EU27_Batteries</t>
+  </si>
   <si>
     <t>Technologies</t>
   </si>
@@ -150,105 +318,6 @@
   </si>
   <si>
     <t>EU27.Batteries</t>
-  </si>
-  <si>
-    <t>Param</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Start Year y0</t>
-  </si>
-  <si>
-    <t>End Year yn</t>
-  </si>
-  <si>
-    <t>hours per year</t>
-  </si>
-  <si>
-    <t>Stf</t>
-  </si>
-  <si>
-    <t>import_EU27_solarPV</t>
-  </si>
-  <si>
-    <t>manufacturing_EU27_solarPV</t>
-  </si>
-  <si>
-    <t>remanufacturing_EU27_solarPV</t>
-  </si>
-  <si>
-    <t>recycling_EU27_solarPV</t>
-  </si>
-  <si>
-    <t>oandm_EU27_solarPV</t>
-  </si>
-  <si>
-    <t>import_EU27_windoff</t>
-  </si>
-  <si>
-    <t>manufacturing_EU27_windoff</t>
-  </si>
-  <si>
-    <t>remanufacturing_EU27_windoff</t>
-  </si>
-  <si>
-    <t>recycling_EU27_windoff</t>
-  </si>
-  <si>
-    <t>oandm_EU27_windoff</t>
-  </si>
-  <si>
-    <t>import_EU27_windon</t>
-  </si>
-  <si>
-    <t>manufacturing_EU27_windon</t>
-  </si>
-  <si>
-    <t>remanufacturing_EU27_windon</t>
-  </si>
-  <si>
-    <t>recycling_EU27_windon</t>
-  </si>
-  <si>
-    <t>oandm_EU27_windon</t>
-  </si>
-  <si>
-    <t>import_EU27_Batteries</t>
-  </si>
-  <si>
-    <t>manufacturing_EU27_Batteries</t>
-  </si>
-  <si>
-    <t>remanufacturing_EU27_Batteries</t>
-  </si>
-  <si>
-    <t>recycling_EU27_Batteries</t>
-  </si>
-  <si>
-    <t>oandm_EU27_Batteries</t>
-  </si>
-  <si>
-    <t>Locations:</t>
-  </si>
-  <si>
-    <t>EU27</t>
-  </si>
-  <si>
-    <t>timestep</t>
-  </si>
-  <si>
-    <t>EU27_solarPV</t>
-  </si>
-  <si>
-    <t>EU27_windoff</t>
-  </si>
-  <si>
-    <t>EU27_windon</t>
-  </si>
-  <si>
-    <t>EU27_Batteries</t>
   </si>
   <si>
     <t>Year</t>
@@ -613,75 +682,6 @@
   <si>
     <t>material_downstream_manufacturing</t>
   </si>
-  <si>
-    <t>solarPV_Polysilicon</t>
-  </si>
-  <si>
-    <t>solarPV_Wafer</t>
-  </si>
-  <si>
-    <t>solarPV_Cell</t>
-  </si>
-  <si>
-    <t>solarPV_Module</t>
-  </si>
-  <si>
-    <t>windon_BladeOn</t>
-  </si>
-  <si>
-    <t>windon_TowerOn</t>
-  </si>
-  <si>
-    <t>windon_NacelleOn</t>
-  </si>
-  <si>
-    <t>windon_AssemblyOn</t>
-  </si>
-  <si>
-    <t>windoff_BladeOff</t>
-  </si>
-  <si>
-    <t>windoff_TowerOff</t>
-  </si>
-  <si>
-    <t>windoff_NacelleOff</t>
-  </si>
-  <si>
-    <t>windoff_AssemblyOff</t>
-  </si>
-  <si>
-    <t>Batteries_CellBatt</t>
-  </si>
-  <si>
-    <t>Batteries_Assembly</t>
-  </si>
-  <si>
-    <t>capex_solarPV_bos</t>
-  </si>
-  <si>
-    <t>capex_windon_bos</t>
-  </si>
-  <si>
-    <t>capex_windoff_bos</t>
-  </si>
-  <si>
-    <t>opexf_solarPV_bos</t>
-  </si>
-  <si>
-    <t>opexf_windon_bos</t>
-  </si>
-  <si>
-    <t>opexf_windoff_bos</t>
-  </si>
-  <si>
-    <t>opexv_solarPV_bos</t>
-  </si>
-  <si>
-    <t>opexv_windon_bos</t>
-  </si>
-  <si>
-    <t>opexv_windoff_bos</t>
-  </si>
 </sst>
 </file>
 
@@ -985,17 +985,17 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
@@ -1055,31 +1055,31 @@
   </cellXfs>
   <cellStyles count="27">
     <cellStyle name="Comma 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Comma 2 2" xfId="23" xr:uid="{FECD9782-8C91-41B4-B84F-82CA16C565D8}"/>
+    <cellStyle name="Comma 2 2" xfId="23" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
     <cellStyle name="Comma 3" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
     <cellStyle name="Komma 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Link" xfId="11" builtinId="8"/>
-    <cellStyle name="Link 2" xfId="13" xr:uid="{846A4194-E7DB-429E-B7E0-05925ADBFEDF}"/>
+    <cellStyle name="Link 2" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
     <cellStyle name="N_CalcSum" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
     <cellStyle name="N_Comment" xfId="8" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
     <cellStyle name="N_Input" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
     <cellStyle name="N_InputCalc" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
     <cellStyle name="N_InputWhite" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="N_Table1_Header" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Normal 10" xfId="26" xr:uid="{CFEEF6FC-564B-4815-9FE1-A319D12A455E}"/>
-    <cellStyle name="Normal 2" xfId="14" xr:uid="{637273B4-B533-4CF1-A6DF-36C96F5F2459}"/>
-    <cellStyle name="Normal 2 2" xfId="25" xr:uid="{A52F4ADB-E42E-44A4-AFE9-6AEED8DEA10E}"/>
-    <cellStyle name="Normal 3" xfId="15" xr:uid="{4F39A1EB-852C-4A00-A443-7D0C5BC04143}"/>
-    <cellStyle name="Normal 4" xfId="16" xr:uid="{2DD131B2-A0B5-42F8-BFBD-C17C1FB4CF36}"/>
-    <cellStyle name="Normal 5" xfId="17" xr:uid="{C49EA547-1505-4E8A-A6C4-F337F54685F5}"/>
-    <cellStyle name="Normal 6" xfId="19" xr:uid="{43856E99-F80A-4029-BF01-2F589682CE08}"/>
-    <cellStyle name="Normal 7" xfId="20" xr:uid="{C557494E-1843-4468-90ED-0552C2DA6780}"/>
-    <cellStyle name="Normal 8" xfId="21" xr:uid="{C4B5DDB4-B623-446C-85D8-1F692A247050}"/>
-    <cellStyle name="Normal 9" xfId="22" xr:uid="{85D86C0B-632A-4484-A2F0-27BE21780E9D}"/>
-    <cellStyle name="Normal 9 2" xfId="24" xr:uid="{2BCB7FF1-58BF-43A9-A31A-6078D9FAEAD7}"/>
-    <cellStyle name="Percent 2" xfId="18" xr:uid="{CDF8E039-4710-41B6-B27B-CBF7686F87C7}"/>
+    <cellStyle name="Normal 10" xfId="26" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
+    <cellStyle name="Normal 2" xfId="14" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="Normal 2 2" xfId="25" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
+    <cellStyle name="Normal 3" xfId="15" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="Normal 4" xfId="16" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="Normal 5" xfId="17" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
+    <cellStyle name="Normal 6" xfId="19" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
+    <cellStyle name="Normal 7" xfId="20" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
+    <cellStyle name="Normal 8" xfId="21" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
+    <cellStyle name="Normal 9" xfId="22" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
+    <cellStyle name="Normal 9 2" xfId="24" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
+    <cellStyle name="Percent 2" xfId="18" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
-    <cellStyle name="Standard 2" xfId="12" xr:uid="{EC6982DB-6FF9-4BB1-84B4-B879E7FD7B13}"/>
+    <cellStyle name="Standard 2" xfId="12" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
     <cellStyle name="Tabelle allgemein" xfId="10" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1093,10 +1093,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1421,15 +1417,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B2">
         <v>2024</v>
@@ -1437,7 +1433,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B3">
         <v>2050</v>
@@ -1445,7 +1441,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="B4">
         <v>730</v>
@@ -1468,16 +1464,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1485,7 +1481,7 @@
         <v>2024</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C2" s="2">
         <v>270613611.10000002</v>
@@ -1497,7 +1493,7 @@
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="25"/>
       <c r="B3" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C3" s="2">
         <v>1047284444</v>
@@ -1510,7 +1506,7 @@
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="25"/>
       <c r="B4" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C4" s="2">
         <v>2930833333</v>
@@ -1522,7 +1518,7 @@
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="26"/>
       <c r="B5" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C5" s="2">
         <v>484006334</v>
@@ -1536,7 +1532,7 @@
         <v>2025</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C6" s="2">
         <v>270613611.10000002</v>
@@ -1548,7 +1544,7 @@
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="25"/>
       <c r="B7" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C7" s="2">
         <v>1047284444</v>
@@ -1560,7 +1556,7 @@
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="25"/>
       <c r="B8" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C8" s="2">
         <v>2930833333</v>
@@ -1572,7 +1568,7 @@
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="26"/>
       <c r="B9" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C9" s="2">
         <f>SUM(C5*(1-0.04052))</f>
@@ -1587,7 +1583,7 @@
         <v>2026</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C10" s="2">
         <v>270613611.10000002</v>
@@ -1599,7 +1595,7 @@
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="25"/>
       <c r="B11" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C11" s="2">
         <v>1047284444</v>
@@ -1611,7 +1607,7 @@
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="25"/>
       <c r="B12" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C12" s="2">
         <v>2930833333</v>
@@ -1623,7 +1619,7 @@
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="26"/>
       <c r="B13" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C13" s="2">
         <f>SUM(C9*(1-0.04052))</f>
@@ -1638,7 +1634,7 @@
         <v>2027</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C14" s="2">
         <v>270613611.10000002</v>
@@ -1650,7 +1646,7 @@
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="25"/>
       <c r="B15" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C15" s="2">
         <v>1047284444</v>
@@ -1662,7 +1658,7 @@
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="25"/>
       <c r="B16" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C16" s="2">
         <v>2930833333</v>
@@ -1674,7 +1670,7 @@
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="26"/>
       <c r="B17" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C17" s="2">
         <f>SUM(C13*(1-0.04052))</f>
@@ -1689,7 +1685,7 @@
         <v>2028</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C18" s="2">
         <v>270613611.10000002</v>
@@ -1701,7 +1697,7 @@
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="25"/>
       <c r="B19" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C19" s="2">
         <v>1047284444</v>
@@ -1713,7 +1709,7 @@
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="25"/>
       <c r="B20" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C20" s="2">
         <v>2930833333</v>
@@ -1725,7 +1721,7 @@
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="26"/>
       <c r="B21" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C21" s="2">
         <f>SUM(C17*(1-0.04052))</f>
@@ -1740,7 +1736,7 @@
         <v>2029</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C22" s="2">
         <v>270613611.10000002</v>
@@ -1752,7 +1748,7 @@
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="25"/>
       <c r="B23" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C23" s="2">
         <v>1047284444</v>
@@ -1764,7 +1760,7 @@
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="25"/>
       <c r="B24" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C24" s="2">
         <v>2930833333</v>
@@ -1776,7 +1772,7 @@
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="26"/>
       <c r="B25" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C25" s="2">
         <f>SUM(C21*(1-0.04052))</f>
@@ -1791,7 +1787,7 @@
         <v>2030</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C26" s="2">
         <v>270613611.10000002</v>
@@ -1803,7 +1799,7 @@
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="25"/>
       <c r="B27" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C27" s="2">
         <v>1047284444</v>
@@ -1815,7 +1811,7 @@
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="25"/>
       <c r="B28" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C28" s="2">
         <v>2930833333</v>
@@ -1827,7 +1823,7 @@
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="26"/>
       <c r="B29" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C29" s="2">
         <f>SUM(C25*(1-0.04052))</f>
@@ -1842,7 +1838,7 @@
         <v>2031</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C30" s="2">
         <v>270613611.10000002</v>
@@ -1854,7 +1850,7 @@
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="25"/>
       <c r="B31" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C31" s="2">
         <v>1047284444</v>
@@ -1866,7 +1862,7 @@
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="25"/>
       <c r="B32" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C32" s="2">
         <v>2930833333</v>
@@ -1878,7 +1874,7 @@
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="26"/>
       <c r="B33" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C33" s="2">
         <f>SUM(C29*(1-0.04052))</f>
@@ -1893,7 +1889,7 @@
         <v>2032</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C34" s="2">
         <v>270613611.10000002</v>
@@ -1905,7 +1901,7 @@
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="25"/>
       <c r="B35" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C35" s="2">
         <v>1047284444</v>
@@ -1917,7 +1913,7 @@
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="25"/>
       <c r="B36" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C36" s="2">
         <v>2930833333</v>
@@ -1929,7 +1925,7 @@
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="26"/>
       <c r="B37" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C37" s="2">
         <f>SUM(C33*(1-0.04052))</f>
@@ -1944,7 +1940,7 @@
         <v>2033</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C38" s="2">
         <v>270613611.10000002</v>
@@ -1956,7 +1952,7 @@
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="25"/>
       <c r="B39" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C39" s="2">
         <v>1047284444</v>
@@ -1968,7 +1964,7 @@
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="25"/>
       <c r="B40" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C40" s="2">
         <v>2930833333</v>
@@ -1980,7 +1976,7 @@
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="26"/>
       <c r="B41" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C41" s="2">
         <f>SUM(C37*(1-0.04052))</f>
@@ -1995,7 +1991,7 @@
         <v>2034</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C42" s="2">
         <v>270613611.10000002</v>
@@ -2007,7 +2003,7 @@
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="25"/>
       <c r="B43" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C43" s="2">
         <v>1047284444</v>
@@ -2019,7 +2015,7 @@
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="25"/>
       <c r="B44" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C44" s="2">
         <v>2930833333</v>
@@ -2031,7 +2027,7 @@
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="26"/>
       <c r="B45" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C45" s="2">
         <f>SUM(C41*(1-0.04052))</f>
@@ -2046,7 +2042,7 @@
         <v>2035</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C46" s="2">
         <v>270613611.10000002</v>
@@ -2058,7 +2054,7 @@
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="25"/>
       <c r="B47" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C47" s="2">
         <v>1047284444</v>
@@ -2070,7 +2066,7 @@
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="25"/>
       <c r="B48" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C48" s="2">
         <v>2930833333</v>
@@ -2082,7 +2078,7 @@
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="26"/>
       <c r="B49" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C49" s="2">
         <f>SUM(C45*(1-0.04052))</f>
@@ -2097,7 +2093,7 @@
         <v>2036</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C50" s="2">
         <v>270613611.10000002</v>
@@ -2109,7 +2105,7 @@
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="25"/>
       <c r="B51" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C51" s="2">
         <v>1047284444</v>
@@ -2121,7 +2117,7 @@
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="25"/>
       <c r="B52" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C52" s="2">
         <v>2930833333</v>
@@ -2133,7 +2129,7 @@
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="26"/>
       <c r="B53" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C53" s="2">
         <f>SUM(C49*(1-0.04052))</f>
@@ -2148,7 +2144,7 @@
         <v>2037</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C54" s="2">
         <v>270613611.10000002</v>
@@ -2160,7 +2156,7 @@
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="25"/>
       <c r="B55" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C55" s="2">
         <v>1047284444</v>
@@ -2172,7 +2168,7 @@
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="25"/>
       <c r="B56" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C56" s="2">
         <v>2930833333</v>
@@ -2184,7 +2180,7 @@
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="26"/>
       <c r="B57" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C57" s="2">
         <f>SUM(C53*(1-0.04052))</f>
@@ -2199,7 +2195,7 @@
         <v>2038</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C58" s="2">
         <v>270613611.10000002</v>
@@ -2211,7 +2207,7 @@
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="25"/>
       <c r="B59" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C59" s="2">
         <v>1047284444</v>
@@ -2223,7 +2219,7 @@
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="25"/>
       <c r="B60" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C60" s="2">
         <v>2930833333</v>
@@ -2235,7 +2231,7 @@
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="26"/>
       <c r="B61" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C61" s="2">
         <f>SUM(C57*(1-0.04052))</f>
@@ -2250,7 +2246,7 @@
         <v>2039</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C62" s="2">
         <v>270613611.10000002</v>
@@ -2262,7 +2258,7 @@
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="25"/>
       <c r="B63" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C63" s="2">
         <v>1047284444</v>
@@ -2274,7 +2270,7 @@
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="25"/>
       <c r="B64" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C64" s="2">
         <v>2930833333</v>
@@ -2286,7 +2282,7 @@
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="26"/>
       <c r="B65" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C65" s="2">
         <f>SUM(C61*(1-0.04052))</f>
@@ -2301,7 +2297,7 @@
         <v>2040</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C66" s="2">
         <v>270613611.10000002</v>
@@ -2313,7 +2309,7 @@
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="25"/>
       <c r="B67" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C67" s="2">
         <v>1047284444</v>
@@ -2325,7 +2321,7 @@
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="25"/>
       <c r="B68" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C68" s="2">
         <v>2930833333</v>
@@ -2337,7 +2333,7 @@
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="26"/>
       <c r="B69" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C69" s="2">
         <f>SUM(C65*(1-0.04052))</f>
@@ -2352,7 +2348,7 @@
         <v>2041</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C70" s="2">
         <v>270613611.10000002</v>
@@ -2364,7 +2360,7 @@
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="25"/>
       <c r="B71" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C71" s="2">
         <v>1047284444</v>
@@ -2376,7 +2372,7 @@
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="25"/>
       <c r="B72" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C72" s="2">
         <v>2930833333</v>
@@ -2388,7 +2384,7 @@
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="26"/>
       <c r="B73" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C73" s="2">
         <f>SUM(C69*(1-0.04052))</f>
@@ -2403,7 +2399,7 @@
         <v>2042</v>
       </c>
       <c r="B74" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C74" s="2">
         <v>270613611.10000002</v>
@@ -2415,7 +2411,7 @@
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="25"/>
       <c r="B75" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C75" s="2">
         <v>1047284444</v>
@@ -2427,7 +2423,7 @@
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="25"/>
       <c r="B76" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C76" s="2">
         <v>2930833333</v>
@@ -2439,7 +2435,7 @@
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="26"/>
       <c r="B77" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C77" s="2">
         <f>SUM(C73*(1-0.04052))</f>
@@ -2454,7 +2450,7 @@
         <v>2043</v>
       </c>
       <c r="B78" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C78" s="2">
         <v>270613611.10000002</v>
@@ -2466,7 +2462,7 @@
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="25"/>
       <c r="B79" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C79" s="2">
         <v>1047284444</v>
@@ -2478,7 +2474,7 @@
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="25"/>
       <c r="B80" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C80" s="2">
         <v>2930833333</v>
@@ -2490,7 +2486,7 @@
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="26"/>
       <c r="B81" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C81" s="2">
         <f>SUM(C77*(1-0.04052))</f>
@@ -2505,7 +2501,7 @@
         <v>2044</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C82" s="2">
         <v>270613611.10000002</v>
@@ -2517,7 +2513,7 @@
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="25"/>
       <c r="B83" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C83" s="2">
         <v>1047284444</v>
@@ -2529,7 +2525,7 @@
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="25"/>
       <c r="B84" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C84" s="2">
         <v>2930833333</v>
@@ -2541,7 +2537,7 @@
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="26"/>
       <c r="B85" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C85" s="2">
         <f>SUM(C81*(1-0.04052))</f>
@@ -2556,7 +2552,7 @@
         <v>2045</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C86" s="2">
         <v>270613611.10000002</v>
@@ -2568,7 +2564,7 @@
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="25"/>
       <c r="B87" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C87" s="2">
         <v>1047284444</v>
@@ -2580,7 +2576,7 @@
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="25"/>
       <c r="B88" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C88" s="2">
         <v>2930833333</v>
@@ -2592,7 +2588,7 @@
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="26"/>
       <c r="B89" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C89" s="2">
         <f>SUM(C85*(1-0.04052))</f>
@@ -2607,7 +2603,7 @@
         <v>2046</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C90" s="2">
         <v>270613611.10000002</v>
@@ -2619,7 +2615,7 @@
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="25"/>
       <c r="B91" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C91" s="2">
         <v>1047284444</v>
@@ -2631,7 +2627,7 @@
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="25"/>
       <c r="B92" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C92" s="2">
         <v>2930833333</v>
@@ -2643,7 +2639,7 @@
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="26"/>
       <c r="B93" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C93" s="2">
         <f>SUM(C89*(1-0.04052))</f>
@@ -2658,7 +2654,7 @@
         <v>2047</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C94" s="2">
         <v>270613611.10000002</v>
@@ -2670,7 +2666,7 @@
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="25"/>
       <c r="B95" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C95" s="2">
         <v>1047284444</v>
@@ -2682,7 +2678,7 @@
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="25"/>
       <c r="B96" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C96" s="2">
         <v>2930833333</v>
@@ -2694,7 +2690,7 @@
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="26"/>
       <c r="B97" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C97" s="2">
         <f>SUM(C93*(1-0.04052))</f>
@@ -2709,7 +2705,7 @@
         <v>2048</v>
       </c>
       <c r="B98" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C98" s="2">
         <v>270613611.10000002</v>
@@ -2721,7 +2717,7 @@
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="25"/>
       <c r="B99" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C99" s="2">
         <v>1047284444</v>
@@ -2733,7 +2729,7 @@
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="25"/>
       <c r="B100" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C100" s="2">
         <v>2930833333</v>
@@ -2745,7 +2741,7 @@
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="26"/>
       <c r="B101" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C101" s="2">
         <f>SUM(C97*(1-0.04052))</f>
@@ -2760,7 +2756,7 @@
         <v>2049</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C102" s="2">
         <v>270613611.10000002</v>
@@ -2772,7 +2768,7 @@
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="25"/>
       <c r="B103" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C103" s="2">
         <v>1047284444</v>
@@ -2784,7 +2780,7 @@
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="25"/>
       <c r="B104" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C104" s="2">
         <v>2930833333</v>
@@ -2796,7 +2792,7 @@
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="26"/>
       <c r="B105" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C105" s="2">
         <f>SUM(C101*(1-0.04052))</f>
@@ -2811,7 +2807,7 @@
         <v>2050</v>
       </c>
       <c r="B106" s="11" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C106" s="2">
         <v>270613611.10000002</v>
@@ -2823,7 +2819,7 @@
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="25"/>
       <c r="B107" s="11" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C107" s="2">
         <v>1047284444</v>
@@ -2835,7 +2831,7 @@
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="25"/>
       <c r="B108" s="11" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C108" s="2">
         <v>2930833333</v>
@@ -2847,7 +2843,7 @@
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="26"/>
       <c r="B109" s="11" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C109" s="2">
         <f>SUM(C105*(1-0.04052))</f>
@@ -2858,35 +2854,34 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B109" xr:uid="{00000000-0009-0000-0000-000009000000}"/>
   <mergeCells count="27">
     <mergeCell ref="A106:A109"/>
+    <mergeCell ref="A62:A65"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A38:A41"/>
     <mergeCell ref="A34:A37"/>
     <mergeCell ref="A82:A85"/>
     <mergeCell ref="A58:A61"/>
     <mergeCell ref="A98:A101"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A94:A97"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A74:A77"/>
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="A42:A45"/>
     <mergeCell ref="A14:A17"/>
     <mergeCell ref="A10:A13"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A86:A89"/>
     <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A46:A49"/>
     <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A94:A97"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A50:A53"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2899,39 +2894,39 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B1" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="C1" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="D1" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="E1" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="F1" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="G1" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="H1" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -2948,13 +2943,13 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C3" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -2971,13 +2966,13 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C4" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -2994,13 +2989,13 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -3015,18 +3010,18 @@
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C6" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -3041,18 +3036,18 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -3067,18 +3062,18 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C8" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -3093,18 +3088,18 @@
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B9" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C9" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -3119,18 +3114,18 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C10" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -3145,18 +3140,18 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C11" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -3173,13 +3168,13 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -3196,13 +3191,13 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B13" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C13" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -3219,13 +3214,13 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B14" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="C14" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -3242,13 +3237,13 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B15" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="C15" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -3263,7 +3258,7 @@
         <v>1</v>
       </c>
       <c r="H15" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -3283,33 +3278,33 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="B1" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="C1" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="D1" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="E1" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="F1" t="s">
-        <v>107</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="D2" s="12">
         <v>11.08059701492537</v>
@@ -3323,13 +3318,13 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="D3" s="12">
         <v>46.4</v>
@@ -3343,13 +3338,13 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="D4" s="12">
         <v>7.6179104477611936</v>
@@ -3363,13 +3358,13 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="D5" s="12">
         <v>0.62328358208955215</v>
@@ -3383,13 +3378,13 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="D6" s="12">
         <v>2.0776119402985072E-2</v>
@@ -3403,13 +3398,13 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="D7" s="12">
         <v>3.047164179104477</v>
@@ -3423,13 +3418,13 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="D8" s="12">
         <v>0.20776119402985069</v>
@@ -3443,13 +3438,13 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="D9" s="12">
         <v>15</v>
@@ -3463,13 +3458,13 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="D10" s="12">
         <v>180</v>
@@ -3483,13 +3478,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="D11" s="12">
         <v>0.80645121600000003</v>
@@ -3498,18 +3493,18 @@
         <v>0.80645121600000003</v>
       </c>
       <c r="F11" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="D12" s="12">
         <v>2.441776000000001E-3</v>
@@ -3518,18 +3513,18 @@
         <v>2.441776000000001E-3</v>
       </c>
       <c r="F12" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="D13" s="12">
         <v>0.99598527400000014</v>
@@ -3538,18 +3533,18 @@
         <v>0.99598527400000014</v>
       </c>
       <c r="F13" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>118</v>
+        <v>141</v>
       </c>
       <c r="D14" s="12">
         <v>1.88752E-3</v>
@@ -3558,18 +3553,18 @@
         <v>1.88752E-3</v>
       </c>
       <c r="F14" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="D15" s="12">
         <v>4.4819000000000013E-5</v>
@@ -3578,18 +3573,18 @@
         <v>4.4819000000000013E-5</v>
       </c>
       <c r="F15" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="D16" s="12">
         <v>4.6005630000000002E-3</v>
@@ -3598,18 +3593,18 @@
         <v>4.6005630000000002E-3</v>
       </c>
       <c r="F16" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="D17" s="12">
         <v>9.0565300000000008E-4</v>
@@ -3618,18 +3613,18 @@
         <v>9.0565300000000008E-4</v>
       </c>
       <c r="F17" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="D18" s="12">
         <v>1.9774658839999999</v>
@@ -3638,18 +3633,18 @@
         <v>1.9774658839999999</v>
       </c>
       <c r="F18" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="D19" s="12">
         <v>3.9663748000000013E-2</v>
@@ -3658,18 +3653,18 @@
         <v>3.9663748000000013E-2</v>
       </c>
       <c r="F19" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="D20" s="12">
         <v>2.1210528160000002</v>
@@ -3678,18 +3673,18 @@
         <v>2.1210528160000002</v>
       </c>
       <c r="F20" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="D21" s="12">
         <v>3.0464199999999999E-4</v>
@@ -3698,18 +3693,18 @@
         <v>3.0464199999999999E-4</v>
       </c>
       <c r="F21" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="D22" s="12">
         <v>5.3289600000000004E-4</v>
@@ -3718,18 +3713,18 @@
         <v>5.3289600000000004E-4</v>
       </c>
       <c r="F22" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="D23" s="12">
         <v>2.3000000000000001E-8</v>
@@ -3738,18 +3733,18 @@
         <v>2.3000000000000001E-8</v>
       </c>
       <c r="F23" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="D24" s="12">
         <v>5.0735241E-2</v>
@@ -3758,18 +3753,18 @@
         <v>5.0735241E-2</v>
       </c>
       <c r="F24" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="D25" s="12">
         <v>1.5200000000000001E-7</v>
@@ -3778,18 +3773,18 @@
         <v>1.5200000000000001E-7</v>
       </c>
       <c r="F25" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="D26" s="12">
         <v>30</v>
@@ -3803,13 +3798,13 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="D27" s="12">
         <v>250</v>
@@ -3823,13 +3818,13 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="D28" s="12">
         <v>0.76185761500000004</v>
@@ -3838,18 +3833,18 @@
         <v>0.76185761500000004</v>
       </c>
       <c r="F28" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="D29" s="12">
         <v>2.0542469999999991E-3</v>
@@ -3858,18 +3853,18 @@
         <v>2.0542469999999991E-3</v>
       </c>
       <c r="F29" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="D30" s="12">
         <v>1.331902E-3</v>
@@ -3878,18 +3873,18 @@
         <v>1.331902E-3</v>
       </c>
       <c r="F30" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="D31" s="12">
         <v>1.553453376</v>
@@ -3898,18 +3893,18 @@
         <v>1.553453376</v>
       </c>
       <c r="F31" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>118</v>
+        <v>141</v>
       </c>
       <c r="D32" s="12">
         <v>6.5629390000000003E-3</v>
@@ -3918,18 +3913,18 @@
         <v>6.5629390000000003E-3</v>
       </c>
       <c r="F32" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="D33" s="12">
         <v>1.592E-5</v>
@@ -3938,18 +3933,18 @@
         <v>1.592E-5</v>
       </c>
       <c r="F33" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="D34" s="12">
         <v>6.3938059999999993E-3</v>
@@ -3958,18 +3953,18 @@
         <v>6.3938059999999993E-3</v>
       </c>
       <c r="F34" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="D35" s="12">
         <v>1.265682E-3</v>
@@ -3978,18 +3973,18 @@
         <v>1.265682E-3</v>
       </c>
       <c r="F35" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="D36" s="12">
         <v>1.0573537260000001</v>
@@ -3998,18 +3993,18 @@
         <v>1.0573537260000001</v>
       </c>
       <c r="F36" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="D37" s="12">
         <v>3.7349900000000001E-4</v>
@@ -4018,18 +4013,18 @@
         <v>3.7349900000000001E-4</v>
       </c>
       <c r="F37" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="D38" s="12">
         <v>0.10560918699999999</v>
@@ -4038,18 +4033,18 @@
         <v>0.10560918699999999</v>
       </c>
       <c r="F38" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="D39" s="12">
         <v>0.86241605300000002</v>
@@ -4058,18 +4053,18 @@
         <v>0.86241605300000002</v>
       </c>
       <c r="F39" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="D40" s="12">
         <v>1.59808E-4</v>
@@ -4078,18 +4073,18 @@
         <v>1.59808E-4</v>
       </c>
       <c r="F40" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="D41" s="12">
         <v>4.3179210000000003E-2</v>
@@ -4098,18 +4093,18 @@
         <v>4.3179210000000003E-2</v>
       </c>
       <c r="F41" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="D42" s="12">
         <v>3.7350900000000011E-4</v>
@@ -4118,18 +4113,18 @@
         <v>3.7350900000000011E-4</v>
       </c>
       <c r="F42" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="D43" s="12">
         <v>2.6648077999999999E-2</v>
@@ -4138,18 +4133,18 @@
         <v>2.6648077999999999E-2</v>
       </c>
       <c r="F43" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="D44" s="12">
         <v>4.3999999999999997E-8</v>
@@ -4158,18 +4153,18 @@
         <v>4.3999999999999997E-8</v>
       </c>
       <c r="F44" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="B45" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="D45">
         <v>0</v>
@@ -4183,13 +4178,13 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="B46" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="C46" s="18" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="D46">
         <v>0</v>
@@ -4214,45 +4209,45 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B1" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="C1" t="s">
-        <v>134</v>
+        <v>157</v>
       </c>
       <c r="D1" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="E1" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="F1" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="G1" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
       <c r="H1" t="s">
-        <v>139</v>
+        <v>162</v>
       </c>
       <c r="I1" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="J1" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="K1" t="s">
-        <v>142</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -4284,10 +4279,10 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -4319,10 +4314,10 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C4">
         <v>365.87143333333341</v>
@@ -4354,10 +4349,10 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -4404,36 +4399,36 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>143</v>
+        <v>166</v>
       </c>
       <c r="B1" t="s">
-        <v>144</v>
+        <v>167</v>
       </c>
       <c r="C1" t="s">
-        <v>145</v>
+        <v>168</v>
       </c>
       <c r="D1" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="E1" t="s">
-        <v>147</v>
+        <v>170</v>
       </c>
       <c r="F1" t="s">
-        <v>148</v>
+        <v>171</v>
       </c>
       <c r="G1" t="s">
-        <v>149</v>
+        <v>172</v>
       </c>
       <c r="H1" t="s">
-        <v>150</v>
+        <v>173</v>
       </c>
       <c r="I1" t="s">
-        <v>151</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="B2">
         <v>227523.06210000001</v>
@@ -4464,7 +4459,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="B3">
         <v>1090137.72</v>
@@ -4495,7 +4490,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="B4">
         <v>189432.22750000001</v>
@@ -4526,7 +4521,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="B5">
         <v>94712.809810000006</v>
@@ -4557,7 +4552,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="B6">
         <v>541.22898280000004</v>
@@ -4588,7 +4583,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="B7">
         <v>58452.73014</v>
@@ -4619,7 +4614,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="B8">
         <v>143</v>
@@ -4650,7 +4645,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>118</v>
+        <v>141</v>
       </c>
       <c r="B9">
         <v>57.291095110000001</v>
@@ -4681,7 +4676,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="B10">
         <v>3.2587681910000001</v>
@@ -4712,7 +4707,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="B11">
         <v>1068</v>
@@ -4743,7 +4738,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="B12">
         <v>133</v>
@@ -4774,7 +4769,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="B13">
         <v>9206.9589369999994</v>
@@ -4805,7 +4800,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="B14">
         <v>512.35706370000003</v>
@@ -4836,7 +4831,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="B15">
         <v>3774.5654399999999</v>
@@ -4867,7 +4862,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="B16">
         <v>999999</v>
@@ -4898,7 +4893,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="B17">
         <v>83.438261490000002</v>
@@ -4929,7 +4924,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="B18">
         <v>19.865756780000002</v>
@@ -4960,7 +4955,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="B19">
         <v>999999</v>
@@ -4991,7 +4986,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="B20">
         <v>999999</v>
@@ -5022,7 +5017,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="B21">
         <v>13.73426465</v>
@@ -5053,7 +5048,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="B22">
         <v>1038.9856569999999</v>
@@ -5084,7 +5079,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="B23">
         <v>999999</v>
@@ -5115,7 +5110,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="B24">
         <v>999999</v>
@@ -5146,7 +5141,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="B25">
         <v>999999</v>
@@ -5177,7 +5172,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="B26">
         <v>999999</v>
@@ -5218,82 +5213,82 @@
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="C1" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="D1" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
       <c r="E1" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="F1" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="G1" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
       <c r="H1" t="s">
-        <v>157</v>
+        <v>180</v>
       </c>
       <c r="I1" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="J1" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="K1" t="s">
-        <v>160</v>
+        <v>183</v>
       </c>
       <c r="L1" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
       <c r="M1" t="s">
-        <v>162</v>
+        <v>185</v>
       </c>
       <c r="N1" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="O1" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="P1" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="Q1" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="R1" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
       <c r="S1" t="s">
-        <v>168</v>
+        <v>191</v>
       </c>
       <c r="T1" t="s">
-        <v>169</v>
+        <v>192</v>
       </c>
       <c r="U1" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="V1" t="s">
-        <v>171</v>
+        <v>194</v>
       </c>
       <c r="W1" t="s">
-        <v>172</v>
+        <v>195</v>
       </c>
       <c r="X1" t="s">
-        <v>173</v>
+        <v>196</v>
       </c>
       <c r="Y1" t="s">
-        <v>174</v>
+        <v>197</v>
       </c>
       <c r="Z1" t="s">
-        <v>175</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
@@ -7468,82 +7463,82 @@
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="C1" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="D1" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
       <c r="E1" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="F1" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="G1" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
       <c r="H1" t="s">
-        <v>157</v>
+        <v>180</v>
       </c>
       <c r="I1" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="J1" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="K1" t="s">
-        <v>160</v>
+        <v>183</v>
       </c>
       <c r="L1" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
       <c r="M1" t="s">
-        <v>162</v>
+        <v>185</v>
       </c>
       <c r="N1" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="O1" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="P1" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="Q1" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="R1" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
       <c r="S1" t="s">
-        <v>168</v>
+        <v>191</v>
       </c>
       <c r="T1" t="s">
-        <v>169</v>
+        <v>192</v>
       </c>
       <c r="U1" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="V1" t="s">
-        <v>171</v>
+        <v>194</v>
       </c>
       <c r="W1" t="s">
-        <v>172</v>
+        <v>195</v>
       </c>
       <c r="X1" t="s">
-        <v>173</v>
+        <v>196</v>
       </c>
       <c r="Y1" t="s">
-        <v>174</v>
+        <v>197</v>
       </c>
       <c r="Z1" t="s">
-        <v>175</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
@@ -9718,82 +9713,82 @@
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="C1" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="D1" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
       <c r="E1" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="F1" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="G1" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
       <c r="H1" t="s">
-        <v>157</v>
+        <v>180</v>
       </c>
       <c r="I1" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="J1" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="K1" t="s">
-        <v>160</v>
+        <v>183</v>
       </c>
       <c r="L1" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
       <c r="M1" t="s">
-        <v>162</v>
+        <v>185</v>
       </c>
       <c r="N1" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="O1" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="P1" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="Q1" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="R1" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
       <c r="S1" t="s">
-        <v>168</v>
+        <v>191</v>
       </c>
       <c r="T1" t="s">
-        <v>169</v>
+        <v>192</v>
       </c>
       <c r="U1" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="V1" t="s">
-        <v>171</v>
+        <v>194</v>
       </c>
       <c r="W1" t="s">
-        <v>172</v>
+        <v>195</v>
       </c>
       <c r="X1" t="s">
-        <v>173</v>
+        <v>196</v>
       </c>
       <c r="Y1" t="s">
-        <v>174</v>
+        <v>197</v>
       </c>
       <c r="Z1" t="s">
-        <v>175</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
@@ -11968,82 +11963,82 @@
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="C1" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="D1" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
       <c r="E1" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="F1" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="G1" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
       <c r="H1" t="s">
-        <v>157</v>
+        <v>180</v>
       </c>
       <c r="I1" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="J1" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="K1" t="s">
-        <v>160</v>
+        <v>183</v>
       </c>
       <c r="L1" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
       <c r="M1" t="s">
-        <v>162</v>
+        <v>185</v>
       </c>
       <c r="N1" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="O1" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="P1" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="Q1" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="R1" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
       <c r="S1" t="s">
-        <v>168</v>
+        <v>191</v>
       </c>
       <c r="T1" t="s">
-        <v>169</v>
+        <v>192</v>
       </c>
       <c r="U1" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="V1" t="s">
-        <v>171</v>
+        <v>194</v>
       </c>
       <c r="W1" t="s">
-        <v>172</v>
+        <v>195</v>
       </c>
       <c r="X1" t="s">
-        <v>173</v>
+        <v>196</v>
       </c>
       <c r="Y1" t="s">
-        <v>174</v>
+        <v>197</v>
       </c>
       <c r="Z1" t="s">
-        <v>175</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
@@ -14218,82 +14213,82 @@
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="C1" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="D1" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
       <c r="E1" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="F1" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="G1" t="s">
+        <v>179</v>
+      </c>
+      <c r="H1" t="s">
+        <v>180</v>
+      </c>
+      <c r="I1" t="s">
+        <v>181</v>
+      </c>
+      <c r="J1" t="s">
+        <v>182</v>
+      </c>
+      <c r="K1" t="s">
+        <v>183</v>
+      </c>
+      <c r="L1" t="s">
+        <v>184</v>
+      </c>
+      <c r="M1" t="s">
+        <v>185</v>
+      </c>
+      <c r="N1" t="s">
+        <v>186</v>
+      </c>
+      <c r="O1" t="s">
+        <v>187</v>
+      </c>
+      <c r="P1" t="s">
+        <v>188</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>189</v>
+      </c>
+      <c r="R1" t="s">
+        <v>190</v>
+      </c>
+      <c r="S1" t="s">
+        <v>191</v>
+      </c>
+      <c r="T1" t="s">
+        <v>192</v>
+      </c>
+      <c r="U1" t="s">
+        <v>193</v>
+      </c>
+      <c r="V1" t="s">
+        <v>194</v>
+      </c>
+      <c r="W1" t="s">
+        <v>195</v>
+      </c>
+      <c r="X1" t="s">
+        <v>196</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>197</v>
+      </c>
+      <c r="Z1" t="s">
         <v>156</v>
-      </c>
-      <c r="H1" t="s">
-        <v>157</v>
-      </c>
-      <c r="I1" t="s">
-        <v>158</v>
-      </c>
-      <c r="J1" t="s">
-        <v>159</v>
-      </c>
-      <c r="K1" t="s">
-        <v>160</v>
-      </c>
-      <c r="L1" t="s">
-        <v>161</v>
-      </c>
-      <c r="M1" t="s">
-        <v>162</v>
-      </c>
-      <c r="N1" t="s">
-        <v>163</v>
-      </c>
-      <c r="O1" t="s">
-        <v>164</v>
-      </c>
-      <c r="P1" t="s">
-        <v>165</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>166</v>
-      </c>
-      <c r="R1" t="s">
-        <v>167</v>
-      </c>
-      <c r="S1" t="s">
-        <v>168</v>
-      </c>
-      <c r="T1" t="s">
-        <v>169</v>
-      </c>
-      <c r="U1" t="s">
-        <v>170</v>
-      </c>
-      <c r="V1" t="s">
-        <v>171</v>
-      </c>
-      <c r="W1" t="s">
-        <v>172</v>
-      </c>
-      <c r="X1" t="s">
-        <v>173</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>174</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
@@ -16484,67 +16479,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" t="s">
         <v>36</v>
       </c>
-      <c r="B1" t="s">
+      <c r="J1" t="s">
         <v>37</v>
       </c>
-      <c r="C1" t="s">
+      <c r="K1" t="s">
         <v>38</v>
       </c>
-      <c r="D1" t="s">
+      <c r="L1" t="s">
         <v>39</v>
       </c>
-      <c r="E1" t="s">
+      <c r="M1" t="s">
         <v>40</v>
       </c>
-      <c r="F1" t="s">
+      <c r="N1" t="s">
         <v>41</v>
       </c>
-      <c r="G1" t="s">
+      <c r="O1" t="s">
         <v>42</v>
       </c>
-      <c r="H1" t="s">
+      <c r="P1" t="s">
         <v>43</v>
       </c>
-      <c r="I1" t="s">
+      <c r="Q1" t="s">
         <v>44</v>
       </c>
-      <c r="J1" t="s">
+      <c r="R1" t="s">
         <v>45</v>
       </c>
-      <c r="K1" t="s">
+      <c r="S1" t="s">
         <v>46</v>
       </c>
-      <c r="L1" t="s">
+      <c r="T1" t="s">
         <v>47</v>
       </c>
-      <c r="M1" t="s">
+      <c r="U1" t="s">
         <v>48</v>
-      </c>
-      <c r="N1" t="s">
-        <v>49</v>
-      </c>
-      <c r="O1" t="s">
-        <v>50</v>
-      </c>
-      <c r="P1" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>52</v>
-      </c>
-      <c r="R1" t="s">
-        <v>53</v>
-      </c>
-      <c r="S1" t="s">
-        <v>54</v>
-      </c>
-      <c r="T1" t="s">
-        <v>55</v>
-      </c>
-      <c r="U1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
@@ -18314,189 +18309,189 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>176</v>
+        <v>199</v>
       </c>
       <c r="B1" t="s">
-        <v>177</v>
+        <v>200</v>
       </c>
       <c r="C1" t="s">
-        <v>178</v>
+        <v>201</v>
       </c>
       <c r="D1" t="s">
-        <v>179</v>
+        <v>202</v>
       </c>
       <c r="E1" t="s">
-        <v>180</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="E2" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="B3" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="C3" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="D3" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="E3" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="B4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C4" t="s">
         <v>88</v>
       </c>
-      <c r="C4" t="s">
-        <v>65</v>
-      </c>
       <c r="D4" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="E4" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="B5" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="D5" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="E5" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D6" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="E6" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B7" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D7" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="E7" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B8" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D8" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="E8" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B9" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D9" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="E9" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D10" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="E10" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="B11" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D11" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="E11" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -18511,28 +18506,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="B1" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="C1" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="D1" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="E1" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="F1" t="s">
-        <v>183</v>
+        <v>206</v>
       </c>
       <c r="G1" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="H1" t="s">
-        <v>184</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -18540,13 +18535,13 @@
         <v>2024</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="E2" s="12">
         <v>64400.000000000007</v>
@@ -18566,13 +18561,13 @@
         <v>2024</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C3" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="D3" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="E3" s="12">
         <v>92000</v>
@@ -18592,13 +18587,13 @@
         <v>2024</v>
       </c>
       <c r="B4" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="D4" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="E4" s="12">
         <v>165600</v>
@@ -18618,13 +18613,13 @@
         <v>2024</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="D5" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="E5" s="12">
         <v>46000</v>
@@ -18644,13 +18639,13 @@
         <v>2024</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D6" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="E6" s="12">
         <v>73600</v>
@@ -18670,13 +18665,13 @@
         <v>2024</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D7" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="E7" s="12">
         <v>82800</v>
@@ -18696,13 +18691,13 @@
         <v>2024</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D8" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="E8" s="12">
         <v>276000</v>
@@ -18722,13 +18717,13 @@
         <v>2024</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D9" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
@@ -18748,13 +18743,13 @@
         <v>2024</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D10" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="E10" s="12">
         <v>165600</v>
@@ -18774,13 +18769,13 @@
         <v>2024</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D11" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="E11" s="12">
         <v>202400</v>
@@ -18800,13 +18795,13 @@
         <v>2024</v>
       </c>
       <c r="B12" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D12" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="E12" s="12">
         <v>202400</v>
@@ -18826,13 +18821,13 @@
         <v>2024</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D13" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="E13" s="12">
         <v>1</v>
@@ -18852,13 +18847,13 @@
         <v>2024</v>
       </c>
       <c r="B14" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C14" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="D14" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -18878,13 +18873,13 @@
         <v>2024</v>
       </c>
       <c r="B15" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C15" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="D15" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -18911,76 +18906,76 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>185</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>186</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>187</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>188</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>189</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>190</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>191</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>192</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>193</v>
+        <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>194</v>
+        <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>196</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>197</v>
+        <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>198</v>
+        <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>199</v>
+        <v>15</v>
       </c>
       <c r="Q1" t="s">
-        <v>200</v>
+        <v>16</v>
       </c>
       <c r="R1" t="s">
-        <v>201</v>
+        <v>17</v>
       </c>
       <c r="S1" t="s">
-        <v>202</v>
+        <v>18</v>
       </c>
       <c r="T1" t="s">
-        <v>203</v>
+        <v>19</v>
       </c>
       <c r="U1" t="s">
-        <v>204</v>
+        <v>20</v>
       </c>
       <c r="V1" t="s">
-        <v>205</v>
+        <v>21</v>
       </c>
       <c r="W1" t="s">
-        <v>206</v>
+        <v>22</v>
       </c>
       <c r="X1" t="s">
-        <v>207</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
@@ -21003,12 +20998,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -21071,22 +21066,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="E1" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="F1" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -27593,90 +27588,90 @@
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1</v>
+        <v>57</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>6</v>
+        <v>62</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>7</v>
+        <v>63</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>67</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>13</v>
+        <v>69</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>14</v>
+        <v>70</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>23</v>
+        <v>79</v>
       </c>
       <c r="Y1" s="4" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="Z1" s="4" t="s">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="AA1" s="4" t="s">
-        <v>26</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>27</v>
+        <v>83</v>
       </c>
       <c r="B2" s="10">
         <v>211115</v>
@@ -27759,7 +27754,7 @@
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="B3" s="7">
         <v>18800</v>
@@ -27842,7 +27837,7 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="B4" s="7">
         <v>195370</v>
@@ -27925,7 +27920,7 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="B5" s="7">
         <v>35000</v>
@@ -28058,19 +28053,19 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="B1" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C1" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D1" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="H1" s="23" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -28466,19 +28461,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -28952,19 +28947,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -29438,19 +29433,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>